<commit_message>
Refactor Excel data handling and improve style caching
- Updated `AddPoolDataToSheet` and `AddPlayerDataToSheet` functions to utilize a cached column name array for metadata, improving performance.
- Enhanced `excel_styles.go` with a caching mechanism for styles to reduce redundant style creation.
- Modified `CreateTagsSheet` to set A4 portrait layout with appropriate margins and row heights, ensuring better label formatting.
- Improved `ApplySeeds` function to use a reverse index for seed-to-player mapping, optimizing collision detection during seed assignments.
- Refactored `CreatePools` and `discoverPool` functions to utilize per-pool sets for dojo and name conflict detection, enhancing efficiency in player assignments.
- Updated tests to reflect changes in pool creation and discovery logic, ensuring robust validation of new functionality.
- Updated example Excel files to reflect changes in formatting and structure.
</commit_message>
<xml_diff>
--- a/playoffs-example-medium.xlsx
+++ b/playoffs-example-medium.xlsx
@@ -19,7 +19,9 @@
     <sheet name="Tree 1" sheetId="10" r:id="rId13"/>
     <sheet name="Tree 2" sheetId="11" r:id="rId14"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName localSheetId="3" name="_xlnm.Print_Area">'Names to Print'!$A$1:$B$48</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -507,7 +509,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -523,6 +525,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -641,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -712,10 +719,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2337,201 +2347,201 @@
     <col customWidth="true" max="2" min="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="E3" s="24" t="s">
+    <row r="6">
+      <c r="E6" s="24" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4">
-      <c r="F4" s="22"/>
-      <c r="G4" s="20"/>
-    </row>
-    <row r="5">
-      <c r="G5" s="21">
+    <row r="7">
+      <c r="F7" s="22"/>
+      <c r="G7" s="20"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="21">
         <v>9</v>
       </c>
     </row>
-    <row r="6">
-      <c r="C6" s="24" t="s">
+    <row r="9">
+      <c r="C9" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="20"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="20"/>
-    </row>
-    <row r="7">
-      <c r="D7" s="22"/>
-      <c r="E7" s="21">
+      <c r="G9" s="20"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="22"/>
+      <c r="E10" s="21">
         <v>1</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="20"/>
-      <c r="I7" s="20"/>
-    </row>
-    <row r="8">
-      <c r="C8" s="24" t="s">
+      <c r="F10" s="23"/>
+      <c r="G10" s="20"/>
+      <c r="I10" s="20"/>
+    </row>
+    <row r="11">
+      <c r="C11" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="20"/>
-      <c r="I8" s="20"/>
-    </row>
-    <row r="9">
-      <c r="I9" s="21">
+      <c r="D11" s="23"/>
+      <c r="E11" s="20"/>
+      <c r="I11" s="20"/>
+    </row>
+    <row r="12">
+      <c r="I12" s="21">
         <v>17</v>
       </c>
     </row>
-    <row r="10">
-      <c r="I10" s="20"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="20"/>
-    </row>
-    <row r="11">
-      <c r="E11" s="24" t="s">
+    <row r="13">
+      <c r="I13" s="20"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="20"/>
+    </row>
+    <row r="14">
+      <c r="E14" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="20"/>
-      <c r="K11" s="20"/>
-    </row>
-    <row r="12">
-      <c r="F12" s="22"/>
-      <c r="G12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="K12" s="20"/>
-    </row>
-    <row r="13">
-      <c r="G13" s="21">
+      <c r="I14" s="20"/>
+      <c r="K14" s="20"/>
+    </row>
+    <row r="15">
+      <c r="F15" s="22"/>
+      <c r="G15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16">
+      <c r="G16" s="21">
         <v>10</v>
       </c>
-      <c r="H13" s="23"/>
-      <c r="I13" s="20"/>
-      <c r="K13" s="20"/>
-    </row>
-    <row r="14">
-      <c r="C14" s="24" t="s">
+      <c r="H16" s="23"/>
+      <c r="I16" s="20"/>
+      <c r="K16" s="20"/>
+    </row>
+    <row r="17">
+      <c r="C17" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="20"/>
-      <c r="K14" s="20"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="22"/>
-      <c r="E15" s="21">
+      <c r="G17" s="20"/>
+      <c r="K17" s="20"/>
+    </row>
+    <row r="18">
+      <c r="D18" s="22"/>
+      <c r="E18" s="21">
         <v>2</v>
       </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="20"/>
-      <c r="K15" s="20"/>
-    </row>
-    <row r="16">
-      <c r="C16" s="24" t="s">
+      <c r="F18" s="23"/>
+      <c r="G18" s="20"/>
+      <c r="K18" s="20"/>
+    </row>
+    <row r="19">
+      <c r="C19" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="20"/>
-      <c r="K16" s="20"/>
-    </row>
-    <row r="17">
-      <c r="K17" s="21">
+      <c r="D19" s="23"/>
+      <c r="E19" s="20"/>
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20">
+      <c r="K20" s="21">
         <v>21</v>
       </c>
     </row>
-    <row r="18">
-      <c r="K18" s="20"/>
-    </row>
-    <row r="19">
-      <c r="E19" s="24" t="s">
+    <row r="21">
+      <c r="K21" s="20"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="K19" s="20"/>
-    </row>
-    <row r="20">
-      <c r="F20" s="22"/>
-      <c r="G20" s="20"/>
-      <c r="K20" s="20"/>
-    </row>
-    <row r="21">
-      <c r="G21" s="21">
+      <c r="K22" s="20"/>
+    </row>
+    <row r="23">
+      <c r="F23" s="22"/>
+      <c r="G23" s="20"/>
+      <c r="K23" s="20"/>
+    </row>
+    <row r="24">
+      <c r="G24" s="21">
         <v>11</v>
       </c>
-      <c r="K21" s="20"/>
-    </row>
-    <row r="22">
-      <c r="C22" s="24" t="s">
+      <c r="K24" s="20"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="G22" s="20"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="20"/>
-      <c r="K22" s="20"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="22"/>
-      <c r="E23" s="21">
+      <c r="G25" s="20"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="20"/>
+      <c r="K25" s="20"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="22"/>
+      <c r="E26" s="21">
         <v>3</v>
       </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="K23" s="20"/>
-    </row>
-    <row r="24">
-      <c r="C24" s="24" t="s">
+      <c r="F26" s="23"/>
+      <c r="G26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="K26" s="20"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="23"/>
-      <c r="E24" s="20"/>
-      <c r="I24" s="20"/>
-      <c r="K24" s="20"/>
-    </row>
-    <row r="25">
-      <c r="I25" s="21">
+      <c r="D27" s="23"/>
+      <c r="E27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="K27" s="20"/>
+    </row>
+    <row r="28">
+      <c r="I28" s="21">
         <v>18</v>
       </c>
-      <c r="J25" s="23"/>
-      <c r="K25" s="20"/>
-    </row>
-    <row r="26">
-      <c r="I26" s="20"/>
-    </row>
-    <row r="27">
-      <c r="E27" s="24" t="s">
+      <c r="J28" s="23"/>
+      <c r="K28" s="20"/>
+    </row>
+    <row r="29">
+      <c r="I29" s="20"/>
+    </row>
+    <row r="30">
+      <c r="E30" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="I27" s="20"/>
-    </row>
-    <row r="28">
-      <c r="F28" s="22"/>
-      <c r="G28" s="20"/>
-      <c r="I28" s="20"/>
-    </row>
-    <row r="29">
-      <c r="G29" s="21">
+      <c r="I30" s="20"/>
+    </row>
+    <row r="31">
+      <c r="F31" s="22"/>
+      <c r="G31" s="20"/>
+      <c r="I31" s="20"/>
+    </row>
+    <row r="32">
+      <c r="G32" s="21">
         <v>12</v>
       </c>
-      <c r="H29" s="23"/>
-      <c r="I29" s="20"/>
-    </row>
-    <row r="30">
-      <c r="C30" s="24" t="s">
+      <c r="H32" s="23"/>
+      <c r="I32" s="20"/>
+    </row>
+    <row r="33">
+      <c r="C33" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="G30" s="20"/>
-    </row>
-    <row r="31">
-      <c r="D31" s="22"/>
-      <c r="E31" s="21">
+      <c r="G33" s="20"/>
+    </row>
+    <row r="34">
+      <c r="D34" s="22"/>
+      <c r="E34" s="21">
         <v>4</v>
       </c>
-      <c r="F31" s="23"/>
-      <c r="G31" s="20"/>
-    </row>
-    <row r="32">
-      <c r="C32" s="24" t="s">
+      <c r="F34" s="23"/>
+      <c r="G34" s="20"/>
+    </row>
+    <row r="35">
+      <c r="C35" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D32" s="23"/>
-      <c r="E32" s="20"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="20"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="true" verticalCentered="true"/>
@@ -2551,201 +2561,201 @@
     <col customWidth="true" max="2" min="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="E3" s="24" t="s">
+    <row r="6">
+      <c r="E6" s="24" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4">
-      <c r="F4" s="22"/>
-      <c r="G4" s="20"/>
-    </row>
-    <row r="5">
-      <c r="G5" s="21">
+    <row r="7">
+      <c r="F7" s="22"/>
+      <c r="G7" s="20"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="21">
         <v>13</v>
       </c>
     </row>
-    <row r="6">
-      <c r="C6" s="24" t="s">
+    <row r="9">
+      <c r="C9" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="G6" s="20"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="20"/>
-    </row>
-    <row r="7">
-      <c r="D7" s="22"/>
-      <c r="E7" s="21">
+      <c r="G9" s="20"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="22"/>
+      <c r="E10" s="21">
         <v>5</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="20"/>
-      <c r="I7" s="20"/>
-    </row>
-    <row r="8">
-      <c r="C8" s="24" t="s">
+      <c r="F10" s="23"/>
+      <c r="G10" s="20"/>
+      <c r="I10" s="20"/>
+    </row>
+    <row r="11">
+      <c r="C11" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="20"/>
-      <c r="I8" s="20"/>
-    </row>
-    <row r="9">
-      <c r="I9" s="21">
+      <c r="D11" s="23"/>
+      <c r="E11" s="20"/>
+      <c r="I11" s="20"/>
+    </row>
+    <row r="12">
+      <c r="I12" s="21">
         <v>19</v>
       </c>
     </row>
-    <row r="10">
-      <c r="I10" s="20"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="20"/>
-    </row>
-    <row r="11">
-      <c r="E11" s="24" t="s">
+    <row r="13">
+      <c r="I13" s="20"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="20"/>
+    </row>
+    <row r="14">
+      <c r="E14" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="I11" s="20"/>
-      <c r="K11" s="20"/>
-    </row>
-    <row r="12">
-      <c r="F12" s="22"/>
-      <c r="G12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="K12" s="20"/>
-    </row>
-    <row r="13">
-      <c r="G13" s="21">
+      <c r="I14" s="20"/>
+      <c r="K14" s="20"/>
+    </row>
+    <row r="15">
+      <c r="F15" s="22"/>
+      <c r="G15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16">
+      <c r="G16" s="21">
         <v>14</v>
       </c>
-      <c r="H13" s="23"/>
-      <c r="I13" s="20"/>
-      <c r="K13" s="20"/>
-    </row>
-    <row r="14">
-      <c r="C14" s="24" t="s">
+      <c r="H16" s="23"/>
+      <c r="I16" s="20"/>
+      <c r="K16" s="20"/>
+    </row>
+    <row r="17">
+      <c r="C17" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="G14" s="20"/>
-      <c r="K14" s="20"/>
-    </row>
-    <row r="15">
-      <c r="D15" s="22"/>
-      <c r="E15" s="21">
+      <c r="G17" s="20"/>
+      <c r="K17" s="20"/>
+    </row>
+    <row r="18">
+      <c r="D18" s="22"/>
+      <c r="E18" s="21">
         <v>6</v>
       </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="20"/>
-      <c r="K15" s="20"/>
-    </row>
-    <row r="16">
-      <c r="C16" s="24" t="s">
+      <c r="F18" s="23"/>
+      <c r="G18" s="20"/>
+      <c r="K18" s="20"/>
+    </row>
+    <row r="19">
+      <c r="C19" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="20"/>
-      <c r="K16" s="20"/>
-    </row>
-    <row r="17">
-      <c r="K17" s="21">
+      <c r="D19" s="23"/>
+      <c r="E19" s="20"/>
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20">
+      <c r="K20" s="21">
         <v>22</v>
       </c>
     </row>
-    <row r="18">
-      <c r="K18" s="20"/>
-    </row>
-    <row r="19">
-      <c r="E19" s="24" t="s">
+    <row r="21">
+      <c r="K21" s="20"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="K19" s="20"/>
-    </row>
-    <row r="20">
-      <c r="F20" s="22"/>
-      <c r="G20" s="20"/>
-      <c r="K20" s="20"/>
-    </row>
-    <row r="21">
-      <c r="G21" s="21">
+      <c r="K22" s="20"/>
+    </row>
+    <row r="23">
+      <c r="F23" s="22"/>
+      <c r="G23" s="20"/>
+      <c r="K23" s="20"/>
+    </row>
+    <row r="24">
+      <c r="G24" s="21">
         <v>15</v>
       </c>
-      <c r="K21" s="20"/>
-    </row>
-    <row r="22">
-      <c r="C22" s="24" t="s">
+      <c r="K24" s="20"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="G22" s="20"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="20"/>
-      <c r="K22" s="20"/>
-    </row>
-    <row r="23">
-      <c r="D23" s="22"/>
-      <c r="E23" s="21">
+      <c r="G25" s="20"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="20"/>
+      <c r="K25" s="20"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="22"/>
+      <c r="E26" s="21">
         <v>7</v>
       </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="K23" s="20"/>
-    </row>
-    <row r="24">
-      <c r="C24" s="24" t="s">
+      <c r="F26" s="23"/>
+      <c r="G26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="K26" s="20"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="23"/>
-      <c r="E24" s="20"/>
-      <c r="I24" s="20"/>
-      <c r="K24" s="20"/>
-    </row>
-    <row r="25">
-      <c r="I25" s="21">
+      <c r="D27" s="23"/>
+      <c r="E27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="K27" s="20"/>
+    </row>
+    <row r="28">
+      <c r="I28" s="21">
         <v>20</v>
       </c>
-      <c r="J25" s="23"/>
-      <c r="K25" s="20"/>
-    </row>
-    <row r="26">
-      <c r="I26" s="20"/>
-    </row>
-    <row r="27">
-      <c r="E27" s="24" t="s">
+      <c r="J28" s="23"/>
+      <c r="K28" s="20"/>
+    </row>
+    <row r="29">
+      <c r="I29" s="20"/>
+    </row>
+    <row r="30">
+      <c r="E30" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="I27" s="20"/>
-    </row>
-    <row r="28">
-      <c r="F28" s="22"/>
-      <c r="G28" s="20"/>
-      <c r="I28" s="20"/>
-    </row>
-    <row r="29">
-      <c r="G29" s="21">
+      <c r="I30" s="20"/>
+    </row>
+    <row r="31">
+      <c r="F31" s="22"/>
+      <c r="G31" s="20"/>
+      <c r="I31" s="20"/>
+    </row>
+    <row r="32">
+      <c r="G32" s="21">
         <v>16</v>
       </c>
-      <c r="H29" s="23"/>
-      <c r="I29" s="20"/>
-    </row>
-    <row r="30">
-      <c r="C30" s="24" t="s">
+      <c r="H32" s="23"/>
+      <c r="I32" s="20"/>
+    </row>
+    <row r="33">
+      <c r="C33" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="G30" s="20"/>
-    </row>
-    <row r="31">
-      <c r="D31" s="22"/>
-      <c r="E31" s="21">
+      <c r="G33" s="20"/>
+    </row>
+    <row r="34">
+      <c r="D34" s="22"/>
+      <c r="E34" s="21">
         <v>8</v>
       </c>
-      <c r="F31" s="23"/>
-      <c r="G31" s="20"/>
-    </row>
-    <row r="32">
-      <c r="C32" s="24" t="s">
+      <c r="F34" s="23"/>
+      <c r="G34" s="20"/>
+    </row>
+    <row r="35">
+      <c r="C35" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="D32" s="23"/>
-      <c r="E32" s="20"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="20"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="true" verticalCentered="true"/>
@@ -3019,46 +3029,46 @@
       <c r="O3" s="27"/>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L4" s="29" t="s">
+      <c r="L4" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="str">
+      <c r="A5" s="28" t="str">
         <f>'data'!$B$3</f>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29" t="str">
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28" t="str">
         <f>'data'!$B$4</f>
       </c>
-      <c r="I5" s="29" t="str">
+      <c r="I5" s="28" t="str">
         <f>'data'!$B$6</f>
       </c>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="29" t="str">
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28" t="str">
         <f>'data'!$B$7</f>
       </c>
     </row>
@@ -3103,46 +3113,46 @@
       <c r="O11" s="27"/>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="D12" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I12" s="28" t="s">
+      <c r="I12" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L12" s="29" t="s">
+      <c r="L12" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O12" t="s">
+      <c r="O12" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="str">
+      <c r="A13" s="28" t="str">
         <f>'data'!$B$9</f>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29" t="str">
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28" t="str">
         <f>'data'!$B$11</f>
       </c>
-      <c r="I13" s="29" t="str">
+      <c r="I13" s="28" t="str">
         <f>'data'!$B$12</f>
       </c>
-      <c r="J13" s="29"/>
-      <c r="K13" s="29"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-      <c r="N13" s="29"/>
-      <c r="O13" s="29" t="str">
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="28"/>
+      <c r="N13" s="28"/>
+      <c r="O13" s="28" t="str">
         <f>'data'!$B$13</f>
       </c>
     </row>
@@ -3187,46 +3197,46 @@
       <c r="O19" s="27"/>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="D20" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I20" s="28" t="s">
+      <c r="I20" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L20" s="29" t="s">
+      <c r="L20" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O20" t="s">
+      <c r="O20" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="str">
+      <c r="A21" s="28" t="str">
         <f>'data'!$B$15</f>
       </c>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29" t="str">
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28" t="str">
         <f>'data'!$B$16</f>
       </c>
-      <c r="I21" s="29" t="str">
+      <c r="I21" s="28" t="str">
         <f>'data'!$B$18</f>
       </c>
-      <c r="J21" s="29"/>
-      <c r="K21" s="29"/>
-      <c r="L21" s="29"/>
-      <c r="M21" s="29"/>
-      <c r="N21" s="29"/>
-      <c r="O21" s="29" t="str">
+      <c r="J21" s="28"/>
+      <c r="K21" s="28"/>
+      <c r="L21" s="28"/>
+      <c r="M21" s="28"/>
+      <c r="N21" s="28"/>
+      <c r="O21" s="28" t="str">
         <f>'data'!$B$19</f>
       </c>
     </row>
@@ -3271,46 +3281,46 @@
       <c r="O27" s="27"/>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I28" s="28" t="s">
+      <c r="I28" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L28" s="29" t="s">
+      <c r="L28" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O28" t="s">
+      <c r="O28" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="29" t="str">
+      <c r="A29" s="28" t="str">
         <f>'data'!$B$21</f>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29" t="str">
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28" t="str">
         <f>'data'!$B$22</f>
       </c>
-      <c r="I29" s="29" t="str">
+      <c r="I29" s="28" t="str">
         <f>'data'!$B$24</f>
       </c>
-      <c r="J29" s="29"/>
-      <c r="K29" s="29"/>
-      <c r="L29" s="29"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="29"/>
-      <c r="O29" s="29" t="str">
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
+      <c r="M29" s="28"/>
+      <c r="N29" s="28"/>
+      <c r="O29" s="28" t="str">
         <f>'data'!$B$25</f>
       </c>
     </row>
@@ -3374,46 +3384,46 @@
       <c r="O42" s="27"/>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="s">
+      <c r="A43" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D43" s="29" t="s">
+      <c r="D43" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I43" s="28" t="s">
+      <c r="I43" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L43" s="29" t="s">
+      <c r="L43" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O43" t="s">
+      <c r="O43" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="str">
+      <c r="A44" s="28" t="str">
         <f>'data'!$B$20</f>
       </c>
-      <c r="B44" s="29"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="29" t="str">
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
+      <c r="G44" s="28" t="str">
         <f>CONCATENATE("M 1 ",'Elimination Matches'!G7)</f>
       </c>
-      <c r="I44" s="29" t="str">
+      <c r="I44" s="28" t="str">
         <f>'data'!$B$5</f>
       </c>
-      <c r="J44" s="29"/>
-      <c r="K44" s="29"/>
-      <c r="L44" s="29"/>
-      <c r="M44" s="29"/>
-      <c r="N44" s="29"/>
-      <c r="O44" s="29" t="str">
+      <c r="J44" s="28"/>
+      <c r="K44" s="28"/>
+      <c r="L44" s="28"/>
+      <c r="M44" s="28"/>
+      <c r="N44" s="28"/>
+      <c r="O44" s="28" t="str">
         <f>CONCATENATE("M 2 ",'Elimination Matches'!O7)</f>
       </c>
     </row>
@@ -3458,46 +3468,46 @@
       <c r="O50" s="27"/>
     </row>
     <row r="51">
-      <c r="A51" s="28" t="s">
+      <c r="A51" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D51" s="29" t="s">
+      <c r="D51" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G51" t="s">
+      <c r="G51" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I51" s="28" t="s">
+      <c r="I51" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L51" s="29" t="s">
+      <c r="L51" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O51" t="s">
+      <c r="O51" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="29" t="str">
+      <c r="A52" s="28" t="str">
         <f>'data'!$B$8</f>
       </c>
-      <c r="B52" s="29"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="29"/>
-      <c r="E52" s="29"/>
-      <c r="F52" s="29"/>
-      <c r="G52" s="29" t="str">
+      <c r="B52" s="28"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="28" t="str">
         <f>CONCATENATE("M 3 ",'Elimination Matches'!G15)</f>
       </c>
-      <c r="I52" s="29" t="str">
+      <c r="I52" s="28" t="str">
         <f>'data'!$B$11</f>
       </c>
-      <c r="J52" s="29"/>
-      <c r="K52" s="29"/>
-      <c r="L52" s="29"/>
-      <c r="M52" s="29"/>
-      <c r="N52" s="29"/>
-      <c r="O52" s="29" t="str">
+      <c r="J52" s="28"/>
+      <c r="K52" s="28"/>
+      <c r="L52" s="28"/>
+      <c r="M52" s="28"/>
+      <c r="N52" s="28"/>
+      <c r="O52" s="28" t="str">
         <f>CONCATENATE("M 4 ",'Elimination Matches'!O15)</f>
       </c>
     </row>
@@ -3542,46 +3552,46 @@
       <c r="O58" s="27"/>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="s">
+      <c r="A59" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D59" s="29" t="s">
+      <c r="D59" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G59" t="s">
+      <c r="G59" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I59" s="28" t="s">
+      <c r="I59" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L59" s="29" t="s">
+      <c r="L59" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O59" t="s">
+      <c r="O59" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="29" t="str">
+      <c r="A60" s="28" t="str">
         <f>'data'!$B$14</f>
       </c>
-      <c r="B60" s="29"/>
-      <c r="C60" s="29"/>
-      <c r="D60" s="29"/>
-      <c r="E60" s="29"/>
-      <c r="F60" s="29"/>
-      <c r="G60" s="29" t="str">
+      <c r="B60" s="28"/>
+      <c r="C60" s="28"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="28"/>
+      <c r="F60" s="28"/>
+      <c r="G60" s="28" t="str">
         <f>CONCATENATE("M 5 ",'Elimination Matches'!G23)</f>
       </c>
-      <c r="I60" s="29" t="str">
+      <c r="I60" s="28" t="str">
         <f>'data'!$B$17</f>
       </c>
-      <c r="J60" s="29"/>
-      <c r="K60" s="29"/>
-      <c r="L60" s="29"/>
-      <c r="M60" s="29"/>
-      <c r="N60" s="29"/>
-      <c r="O60" s="29" t="str">
+      <c r="J60" s="28"/>
+      <c r="K60" s="28"/>
+      <c r="L60" s="28"/>
+      <c r="M60" s="28"/>
+      <c r="N60" s="28"/>
+      <c r="O60" s="28" t="str">
         <f>CONCATENATE("M 6 ",'Elimination Matches'!O23)</f>
       </c>
     </row>
@@ -3626,46 +3636,46 @@
       <c r="O66" s="27"/>
     </row>
     <row r="67">
-      <c r="A67" s="28" t="s">
+      <c r="A67" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D67" s="29" t="s">
+      <c r="D67" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G67" t="s">
+      <c r="G67" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I67" s="28" t="s">
+      <c r="I67" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L67" s="29" t="s">
+      <c r="L67" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O67" t="s">
+      <c r="O67" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="29" t="str">
+      <c r="A68" s="28" t="str">
         <f>'data'!$B$20</f>
       </c>
-      <c r="B68" s="29"/>
-      <c r="C68" s="29"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="29"/>
-      <c r="F68" s="29"/>
-      <c r="G68" s="29" t="str">
+      <c r="B68" s="28"/>
+      <c r="C68" s="28"/>
+      <c r="D68" s="28"/>
+      <c r="E68" s="28"/>
+      <c r="F68" s="28"/>
+      <c r="G68" s="28" t="str">
         <f>CONCATENATE("M 7 ",'Elimination Matches'!G31)</f>
       </c>
-      <c r="I68" s="29" t="str">
+      <c r="I68" s="28" t="str">
         <f>'data'!$B$23</f>
       </c>
-      <c r="J68" s="29"/>
-      <c r="K68" s="29"/>
-      <c r="L68" s="29"/>
-      <c r="M68" s="29"/>
-      <c r="N68" s="29"/>
-      <c r="O68" s="29" t="str">
+      <c r="J68" s="28"/>
+      <c r="K68" s="28"/>
+      <c r="L68" s="28"/>
+      <c r="M68" s="28"/>
+      <c r="N68" s="28"/>
+      <c r="O68" s="28" t="str">
         <f>CONCATENATE("M 8 ",'Elimination Matches'!O31)</f>
       </c>
     </row>
@@ -3729,46 +3739,46 @@
       <c r="O81" s="27"/>
     </row>
     <row r="82">
-      <c r="A82" s="28" t="s">
+      <c r="A82" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D82" s="29" t="s">
+      <c r="D82" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G82" t="s">
+      <c r="G82" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I82" s="28" t="s">
+      <c r="I82" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L82" s="29" t="s">
+      <c r="L82" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O82" t="s">
+      <c r="O82" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="29" t="str">
+      <c r="A83" s="28" t="str">
         <f>CONCATENATE("M 9 ",'Elimination Matches'!G46)</f>
       </c>
-      <c r="B83" s="29"/>
-      <c r="C83" s="29"/>
-      <c r="D83" s="29"/>
-      <c r="E83" s="29"/>
-      <c r="F83" s="29"/>
-      <c r="G83" s="29" t="str">
+      <c r="B83" s="28"/>
+      <c r="C83" s="28"/>
+      <c r="D83" s="28"/>
+      <c r="E83" s="28"/>
+      <c r="F83" s="28"/>
+      <c r="G83" s="28" t="str">
         <f>CONCATENATE("M 10 ",'Elimination Matches'!O46)</f>
       </c>
-      <c r="I83" s="29" t="str">
+      <c r="I83" s="28" t="str">
         <f>CONCATENATE("M 11 ",'Elimination Matches'!G54)</f>
       </c>
-      <c r="J83" s="29"/>
-      <c r="K83" s="29"/>
-      <c r="L83" s="29"/>
-      <c r="M83" s="29"/>
-      <c r="N83" s="29"/>
-      <c r="O83" s="29" t="str">
+      <c r="J83" s="28"/>
+      <c r="K83" s="28"/>
+      <c r="L83" s="28"/>
+      <c r="M83" s="28"/>
+      <c r="N83" s="28"/>
+      <c r="O83" s="28" t="str">
         <f>CONCATENATE("M 12 ",'Elimination Matches'!O54)</f>
       </c>
     </row>
@@ -3813,46 +3823,46 @@
       <c r="O89" s="27"/>
     </row>
     <row r="90">
-      <c r="A90" s="28" t="s">
+      <c r="A90" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D90" s="29" t="s">
+      <c r="D90" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G90" t="s">
+      <c r="G90" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I90" s="28" t="s">
+      <c r="I90" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L90" s="29" t="s">
+      <c r="L90" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O90" t="s">
+      <c r="O90" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="29" t="str">
+      <c r="A91" s="28" t="str">
         <f>CONCATENATE("M 13 ",'Elimination Matches'!G62)</f>
       </c>
-      <c r="B91" s="29"/>
-      <c r="C91" s="29"/>
-      <c r="D91" s="29"/>
-      <c r="E91" s="29"/>
-      <c r="F91" s="29"/>
-      <c r="G91" s="29" t="str">
+      <c r="B91" s="28"/>
+      <c r="C91" s="28"/>
+      <c r="D91" s="28"/>
+      <c r="E91" s="28"/>
+      <c r="F91" s="28"/>
+      <c r="G91" s="28" t="str">
         <f>CONCATENATE("M 14 ",'Elimination Matches'!O62)</f>
       </c>
-      <c r="I91" s="29" t="str">
+      <c r="I91" s="28" t="str">
         <f>CONCATENATE("M 15 ",'Elimination Matches'!G70)</f>
       </c>
-      <c r="J91" s="29"/>
-      <c r="K91" s="29"/>
-      <c r="L91" s="29"/>
-      <c r="M91" s="29"/>
-      <c r="N91" s="29"/>
-      <c r="O91" s="29" t="str">
+      <c r="J91" s="28"/>
+      <c r="K91" s="28"/>
+      <c r="L91" s="28"/>
+      <c r="M91" s="28"/>
+      <c r="N91" s="28"/>
+      <c r="O91" s="28" t="str">
         <f>CONCATENATE("M 16 ",'Elimination Matches'!O70)</f>
       </c>
     </row>
@@ -3916,46 +3926,46 @@
       <c r="O104" s="27"/>
     </row>
     <row r="105">
-      <c r="A105" s="28" t="s">
+      <c r="A105" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D105" s="29" t="s">
+      <c r="D105" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G105" t="s">
+      <c r="G105" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="I105" s="28" t="s">
+      <c r="I105" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="L105" s="29" t="s">
+      <c r="L105" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="O105" t="s">
+      <c r="O105" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="29" t="str">
+      <c r="A106" s="28" t="str">
         <f>CONCATENATE("M 17 ",'Elimination Matches'!G85)</f>
       </c>
-      <c r="B106" s="29"/>
-      <c r="C106" s="29"/>
-      <c r="D106" s="29"/>
-      <c r="E106" s="29"/>
-      <c r="F106" s="29"/>
-      <c r="G106" s="29" t="str">
+      <c r="B106" s="28"/>
+      <c r="C106" s="28"/>
+      <c r="D106" s="28"/>
+      <c r="E106" s="28"/>
+      <c r="F106" s="28"/>
+      <c r="G106" s="28" t="str">
         <f>CONCATENATE("M 18 ",'Elimination Matches'!O85)</f>
       </c>
-      <c r="I106" s="29" t="str">
+      <c r="I106" s="28" t="str">
         <f>CONCATENATE("M 19 ",'Elimination Matches'!G93)</f>
       </c>
-      <c r="J106" s="29"/>
-      <c r="K106" s="29"/>
-      <c r="L106" s="29"/>
-      <c r="M106" s="29"/>
-      <c r="N106" s="29"/>
-      <c r="O106" s="29" t="str">
+      <c r="J106" s="28"/>
+      <c r="K106" s="28"/>
+      <c r="L106" s="28"/>
+      <c r="M106" s="28"/>
+      <c r="N106" s="28"/>
+      <c r="O106" s="28" t="str">
         <f>CONCATENATE("M 20 ",'Elimination Matches'!O93)</f>
       </c>
     </row>
@@ -4010,26 +4020,26 @@
       <c r="G119" s="27"/>
     </row>
     <row r="120">
-      <c r="A120" s="28" t="s">
+      <c r="A120" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D120" s="29" t="s">
+      <c r="D120" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="G120" t="s">
+      <c r="G120" s="30" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="29" t="str">
+      <c r="A121" s="28" t="str">
         <f>CONCATENATE("M 21 ",'Elimination Matches'!G108)</f>
       </c>
-      <c r="B121" s="29"/>
-      <c r="C121" s="29"/>
-      <c r="D121" s="29"/>
-      <c r="E121" s="29"/>
-      <c r="F121" s="29"/>
-      <c r="G121" s="29" t="str">
+      <c r="B121" s="28"/>
+      <c r="C121" s="28"/>
+      <c r="D121" s="28"/>
+      <c r="E121" s="28"/>
+      <c r="F121" s="28"/>
+      <c r="G121" s="28" t="str">
         <f>CONCATENATE("M 22 ",'Elimination Matches'!O108)</f>
       </c>
     </row>
@@ -4088,8 +4098,8 @@
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="115" customHeight="true"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="10" width="21.6640625"/>
-    <col customWidth="true" max="2" min="2" style="9" width="170.6640625"/>
+    <col customWidth="true" max="1" min="1" style="10" width="20"/>
+    <col customWidth="true" max="2" min="2" style="9" width="170"/>
     <col max="16384" min="3" style="8" width="10.83203125"/>
   </cols>
   <sheetData>
@@ -4410,6 +4420,6 @@
   </mergeCells>
   <printOptions horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="0" horizontalDpi="0" orientation="landscape" paperSize="8" verticalDpi="0"/>
+  <pageSetup fitToHeight="0" fitToWidth="1" horizontalDpi="0" orientation="landscape" paperSize="8" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add support for multiple courts (Shiaijo) in playoffs and pools
- Introduced a new `courts` flag in both `create-playoffs` and `create-pools` commands to specify the number of courts.
- Updated playoff and pool creation logic to distribute matches and pools across the specified number of courts.
- Enhanced Excel output to label tree sheets with corresponding Shiaijo names based on the number of courts.
- Implemented helper functions to assign pools to courts and reorder pools for balanced distribution.
- Modified Excel sheet headers and formulas to accommodate the new courts feature.
- Added tests for new functionality, including court assignment and pool reordering.
</commit_message>
<xml_diff>
--- a/playoffs-example-medium.xlsx
+++ b/playoffs-example-medium.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t>Elimination Round 1</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Number of Elimination Matches</t>
+  </si>
+  <si>
+    <t>Title prefix:</t>
   </si>
   <si>
     <t>Number</t>
@@ -483,12 +486,12 @@
     </font>
     <font>
       <family val="2"/>
+      <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="12"/>
     </font>
     <font>
       <family val="2"/>
-      <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="12"/>
     </font>
@@ -597,6 +600,20 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
     </border>
     <border>
       <left style="medium">
@@ -612,20 +629,6 @@
       </top>
     </border>
     <border>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -695,37 +698,37 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="true" applyAlignment="false">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -954,358 +957,360 @@
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+    </row>
+    <row r="2" spans="1:2" ht="12.75" customHeight="true">
+      <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C2" t="s">
         <v>14</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="12.75" customHeight="true">
-      <c r="A2" s="1">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="E2" t="s">
         <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="12.75" customHeight="true">
       <c r="A3" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
         <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="12.75" customHeight="true">
       <c r="A4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
         <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="12.75" customHeight="true">
       <c r="A5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
         <v>25</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="12.75" customHeight="true">
       <c r="A6" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
         <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="12.75" customHeight="true">
       <c r="A7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
         <v>31</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="12.75" customHeight="true">
       <c r="A8" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
         <v>34</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="12.75" customHeight="true">
       <c r="A9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
         <v>37</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="12.75" customHeight="true">
       <c r="A10" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
         <v>40</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="12.75" customHeight="true">
       <c r="A11" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
         <v>43</v>
-      </c>
-      <c r="D11" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="12.75" customHeight="true">
       <c r="A12" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
         <v>44</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>43</v>
-      </c>
-      <c r="D12" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="12.75" customHeight="true">
       <c r="A13">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
         <v>46</v>
-      </c>
-      <c r="C13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="12.75" customHeight="true">
       <c r="A14" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
         <v>49</v>
-      </c>
-      <c r="C14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="12.75" customHeight="true">
       <c r="A15" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
         <v>52</v>
-      </c>
-      <c r="C15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="12.75" customHeight="true">
       <c r="A16" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
         <v>55</v>
-      </c>
-      <c r="C16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="12.75" customHeight="true">
       <c r="A17">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" t="s">
         <v>58</v>
-      </c>
-      <c r="C17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="12.75" customHeight="true">
       <c r="A18" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" t="s">
         <v>61</v>
-      </c>
-      <c r="C18" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="12.75" customHeight="true">
       <c r="A19" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" t="s">
         <v>64</v>
-      </c>
-      <c r="C19" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="12.75" customHeight="true">
       <c r="A20" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" t="s">
         <v>67</v>
-      </c>
-      <c r="C20" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="12.75" customHeight="true">
       <c r="A21">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" t="s">
         <v>19</v>
-      </c>
-      <c r="B21" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D21" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="12.75" customHeight="true">
       <c r="A22" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" t="s">
         <v>72</v>
-      </c>
-      <c r="C22" t="s">
-        <v>73</v>
-      </c>
-      <c r="D22" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="12.75" customHeight="true">
       <c r="A23" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" t="s">
         <v>75</v>
-      </c>
-      <c r="C23" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="12.75" customHeight="true">
       <c r="A24" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" t="s">
         <v>78</v>
-      </c>
-      <c r="C24" t="s">
-        <v>79</v>
-      </c>
-      <c r="D24" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="12.75" customHeight="true">
       <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>79</v>
+      </c>
+      <c r="C25" t="s">
+        <v>80</v>
+      </c>
+      <c r="D25" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="12.75" customHeight="true">
+      <c r="A26" s="1">
         <v>23</v>
       </c>
-      <c r="B25" t="s">
-        <v>81</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="B26" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D25" t="s">
+      <c r="C26" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" ht="12.75" customHeight="true">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
+      <c r="D26" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="27" spans="1:2" ht="12.75" customHeight="true">
       <c r="A27" s="1"/>
@@ -2347,203 +2352,226 @@
     <col customWidth="true" max="2" min="2" width="10"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="str">
+        <f>IF(data!$B$1="","Shiaijo A",data!$B$1&amp;" - Shiaijo A")</f>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+    </row>
     <row r="6">
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="F7" s="23"/>
+      <c r="G7" s="21"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="22">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="21"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="21"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="23"/>
+      <c r="E10" s="22">
+        <v>1</v>
+      </c>
+      <c r="F10" s="24"/>
+      <c r="G10" s="21"/>
+      <c r="I10" s="21"/>
+    </row>
+    <row r="11">
+      <c r="C11" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="21"/>
+      <c r="I11" s="21"/>
+    </row>
+    <row r="12">
+      <c r="I12" s="22">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="I13" s="21"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="21"/>
+    </row>
+    <row r="14">
+      <c r="E14" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="21"/>
+      <c r="K14" s="21"/>
+    </row>
+    <row r="15">
+      <c r="F15" s="23"/>
+      <c r="G15" s="21"/>
+      <c r="I15" s="21"/>
+      <c r="K15" s="21"/>
+    </row>
+    <row r="16">
+      <c r="G16" s="22">
+        <v>10</v>
+      </c>
+      <c r="H16" s="24"/>
+      <c r="I16" s="21"/>
+      <c r="K16" s="21"/>
+    </row>
+    <row r="17">
+      <c r="C17" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="21"/>
+      <c r="K17" s="21"/>
+    </row>
+    <row r="18">
+      <c r="D18" s="23"/>
+      <c r="E18" s="22">
+        <v>2</v>
+      </c>
+      <c r="F18" s="24"/>
+      <c r="G18" s="21"/>
+      <c r="K18" s="21"/>
+    </row>
+    <row r="19">
+      <c r="C19" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="24"/>
+      <c r="E19" s="21"/>
+      <c r="K19" s="21"/>
+    </row>
+    <row r="20">
+      <c r="K20" s="22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="K21" s="21"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="K22" s="21"/>
+    </row>
+    <row r="23">
+      <c r="F23" s="23"/>
+      <c r="G23" s="21"/>
+      <c r="K23" s="21"/>
+    </row>
+    <row r="24">
+      <c r="G24" s="22">
+        <v>11</v>
+      </c>
+      <c r="K24" s="21"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="G25" s="21"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="21"/>
+      <c r="K25" s="21"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="23"/>
+      <c r="E26" s="22">
+        <v>3</v>
+      </c>
+      <c r="F26" s="24"/>
+      <c r="G26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="K26" s="21"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="24"/>
+      <c r="E27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="K27" s="21"/>
+    </row>
+    <row r="28">
+      <c r="I28" s="22">
         <v>18</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="F7" s="22"/>
-      <c r="G7" s="20"/>
-    </row>
-    <row r="8">
-      <c r="G8" s="21">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="C9" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="20"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="22"/>
-      <c r="E10" s="21">
-        <v>1</v>
-      </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="20"/>
-      <c r="I10" s="20"/>
-    </row>
-    <row r="11">
-      <c r="C11" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="20"/>
-      <c r="I11" s="20"/>
-    </row>
-    <row r="12">
-      <c r="I12" s="21">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="I13" s="20"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="20"/>
-    </row>
-    <row r="14">
-      <c r="E14" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="I14" s="20"/>
-      <c r="K14" s="20"/>
-    </row>
-    <row r="15">
-      <c r="F15" s="22"/>
-      <c r="G15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="K15" s="20"/>
-    </row>
-    <row r="16">
-      <c r="G16" s="21">
-        <v>10</v>
-      </c>
-      <c r="H16" s="23"/>
-      <c r="I16" s="20"/>
-      <c r="K16" s="20"/>
-    </row>
-    <row r="17">
-      <c r="C17" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G17" s="20"/>
-      <c r="K17" s="20"/>
-    </row>
-    <row r="18">
-      <c r="D18" s="22"/>
-      <c r="E18" s="21">
-        <v>2</v>
-      </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="20"/>
-      <c r="K18" s="20"/>
-    </row>
-    <row r="19">
-      <c r="C19" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="23"/>
-      <c r="E19" s="20"/>
-      <c r="K19" s="20"/>
-    </row>
-    <row r="20">
-      <c r="K20" s="21">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="K21" s="20"/>
-    </row>
-    <row r="22">
-      <c r="E22" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="K22" s="20"/>
-    </row>
-    <row r="23">
-      <c r="F23" s="22"/>
-      <c r="G23" s="20"/>
-      <c r="K23" s="20"/>
-    </row>
-    <row r="24">
-      <c r="G24" s="21">
-        <v>11</v>
-      </c>
-      <c r="K24" s="20"/>
-    </row>
-    <row r="25">
-      <c r="C25" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="20"/>
-      <c r="K25" s="20"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="22"/>
-      <c r="E26" s="21">
-        <v>3</v>
-      </c>
-      <c r="F26" s="23"/>
-      <c r="G26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="K26" s="20"/>
-    </row>
-    <row r="27">
-      <c r="C27" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="23"/>
-      <c r="E27" s="20"/>
-      <c r="I27" s="20"/>
-      <c r="K27" s="20"/>
-    </row>
-    <row r="28">
-      <c r="I28" s="21">
-        <v>18</v>
-      </c>
-      <c r="J28" s="23"/>
-      <c r="K28" s="20"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="21"/>
     </row>
     <row r="29">
-      <c r="I29" s="20"/>
+      <c r="I29" s="21"/>
     </row>
     <row r="30">
-      <c r="E30" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="I30" s="20"/>
+      <c r="E30" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="I30" s="21"/>
     </row>
     <row r="31">
-      <c r="F31" s="22"/>
-      <c r="G31" s="20"/>
-      <c r="I31" s="20"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="21"/>
+      <c r="I31" s="21"/>
     </row>
     <row r="32">
-      <c r="G32" s="21">
+      <c r="G32" s="22">
         <v>12</v>
       </c>
-      <c r="H32" s="23"/>
-      <c r="I32" s="20"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="21"/>
     </row>
     <row r="33">
-      <c r="C33" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="G33" s="20"/>
+      <c r="C33" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="21"/>
     </row>
     <row r="34">
-      <c r="D34" s="22"/>
-      <c r="E34" s="21">
+      <c r="D34" s="23"/>
+      <c r="E34" s="22">
         <v>4</v>
       </c>
-      <c r="F34" s="23"/>
-      <c r="G34" s="20"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="21"/>
     </row>
     <row r="35">
-      <c r="C35" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D35" s="23"/>
-      <c r="E35" s="20"/>
+      <c r="C35" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" s="24"/>
+      <c r="E35" s="21"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
   <printOptions horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2561,203 +2589,226 @@
     <col customWidth="true" max="2" min="2" width="10"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="str">
+        <f>IF(data!$B$1="","Shiaijo B",data!$B$1&amp;" - Shiaijo B")</f>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+    </row>
     <row r="6">
-      <c r="E6" s="24" t="s">
-        <v>51</v>
+      <c r="E6" s="25" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="7">
-      <c r="F7" s="22"/>
-      <c r="G7" s="20"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="21"/>
     </row>
     <row r="8">
-      <c r="G8" s="21">
+      <c r="G8" s="22">
         <v>13</v>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="20"/>
+      <c r="C9" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="21"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="21"/>
     </row>
     <row r="10">
-      <c r="D10" s="22"/>
-      <c r="E10" s="21">
+      <c r="D10" s="23"/>
+      <c r="E10" s="22">
         <v>5</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="20"/>
-      <c r="I10" s="20"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="21"/>
+      <c r="I10" s="21"/>
     </row>
     <row r="11">
-      <c r="C11" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="20"/>
-      <c r="I11" s="20"/>
+      <c r="C11" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="21"/>
+      <c r="I11" s="21"/>
     </row>
     <row r="12">
-      <c r="I12" s="21">
+      <c r="I12" s="22">
         <v>19</v>
       </c>
     </row>
     <row r="13">
-      <c r="I13" s="20"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="20"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="21"/>
     </row>
     <row r="14">
-      <c r="E14" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="I14" s="20"/>
-      <c r="K14" s="20"/>
+      <c r="E14" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="21"/>
+      <c r="K14" s="21"/>
     </row>
     <row r="15">
-      <c r="F15" s="22"/>
-      <c r="G15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="K15" s="20"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="21"/>
+      <c r="I15" s="21"/>
+      <c r="K15" s="21"/>
     </row>
     <row r="16">
-      <c r="G16" s="21">
+      <c r="G16" s="22">
         <v>14</v>
       </c>
-      <c r="H16" s="23"/>
-      <c r="I16" s="20"/>
-      <c r="K16" s="20"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="21"/>
+      <c r="K16" s="21"/>
     </row>
     <row r="17">
-      <c r="C17" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" s="20"/>
-      <c r="K17" s="20"/>
+      <c r="C17" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" s="21"/>
+      <c r="K17" s="21"/>
     </row>
     <row r="18">
-      <c r="D18" s="22"/>
-      <c r="E18" s="21">
+      <c r="D18" s="23"/>
+      <c r="E18" s="22">
         <v>6</v>
       </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="20"/>
-      <c r="K18" s="20"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="21"/>
+      <c r="K18" s="21"/>
     </row>
     <row r="19">
-      <c r="C19" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="D19" s="23"/>
-      <c r="E19" s="20"/>
-      <c r="K19" s="20"/>
+      <c r="C19" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="24"/>
+      <c r="E19" s="21"/>
+      <c r="K19" s="21"/>
     </row>
     <row r="20">
-      <c r="K20" s="21">
+      <c r="K20" s="22">
         <v>22</v>
       </c>
     </row>
     <row r="21">
-      <c r="K21" s="20"/>
+      <c r="K21" s="21"/>
     </row>
     <row r="22">
-      <c r="E22" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="K22" s="20"/>
+      <c r="E22" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22" s="21"/>
     </row>
     <row r="23">
-      <c r="F23" s="22"/>
-      <c r="G23" s="20"/>
-      <c r="K23" s="20"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="21"/>
+      <c r="K23" s="21"/>
     </row>
     <row r="24">
-      <c r="G24" s="21">
+      <c r="G24" s="22">
         <v>15</v>
       </c>
-      <c r="K24" s="20"/>
+      <c r="K24" s="21"/>
     </row>
     <row r="25">
-      <c r="C25" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="20"/>
-      <c r="K25" s="20"/>
+      <c r="C25" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" s="21"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="21"/>
+      <c r="K25" s="21"/>
     </row>
     <row r="26">
-      <c r="D26" s="22"/>
-      <c r="E26" s="21">
+      <c r="D26" s="23"/>
+      <c r="E26" s="22">
         <v>7</v>
       </c>
-      <c r="F26" s="23"/>
-      <c r="G26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="K26" s="20"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="K26" s="21"/>
     </row>
     <row r="27">
-      <c r="C27" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="D27" s="23"/>
-      <c r="E27" s="20"/>
-      <c r="I27" s="20"/>
-      <c r="K27" s="20"/>
+      <c r="C27" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="24"/>
+      <c r="E27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="K27" s="21"/>
     </row>
     <row r="28">
-      <c r="I28" s="21">
+      <c r="I28" s="22">
         <v>20</v>
       </c>
-      <c r="J28" s="23"/>
-      <c r="K28" s="20"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="21"/>
     </row>
     <row r="29">
-      <c r="I29" s="20"/>
+      <c r="I29" s="21"/>
     </row>
     <row r="30">
-      <c r="E30" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="I30" s="20"/>
+      <c r="E30" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="I30" s="21"/>
     </row>
     <row r="31">
-      <c r="F31" s="22"/>
-      <c r="G31" s="20"/>
-      <c r="I31" s="20"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="21"/>
+      <c r="I31" s="21"/>
     </row>
     <row r="32">
-      <c r="G32" s="21">
+      <c r="G32" s="22">
         <v>16</v>
       </c>
-      <c r="H32" s="23"/>
-      <c r="I32" s="20"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="21"/>
     </row>
     <row r="33">
-      <c r="C33" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="G33" s="20"/>
+      <c r="C33" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G33" s="21"/>
     </row>
     <row r="34">
-      <c r="D34" s="22"/>
-      <c r="E34" s="21">
+      <c r="D34" s="23"/>
+      <c r="E34" s="22">
         <v>8</v>
       </c>
-      <c r="F34" s="23"/>
-      <c r="G34" s="20"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="21"/>
     </row>
     <row r="35">
-      <c r="C35" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="D35" s="23"/>
-      <c r="E35" s="20"/>
+      <c r="C35" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="D35" s="24"/>
+      <c r="E35" s="21"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
   <printOptions horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.25" right="0.25" top="0" bottom="0" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2990,67 +3041,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17" thickBot="true">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="I3" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
-      <c r="O3" s="27"/>
+      <c r="A3" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="I3" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
     </row>
     <row r="4">
       <c r="A4" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D4" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I4" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="L4" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I4" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L4" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O4" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="str">
-        <f>'data'!$B$3</f>
+        <f>'data'!$B$4</f>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28"/>
@@ -3058,10 +3109,10 @@
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
       <c r="G5" s="28" t="str">
-        <f>'data'!$B$4</f>
+        <f>'data'!$B$5</f>
       </c>
       <c r="I5" s="28" t="str">
-        <f>'data'!$B$6</f>
+        <f>'data'!$B$7</f>
       </c>
       <c r="J5" s="28"/>
       <c r="K5" s="28"/>
@@ -3069,72 +3120,72 @@
       <c r="M5" s="28"/>
       <c r="N5" s="28"/>
       <c r="O5" s="28" t="str">
-        <f>'data'!$B$7</f>
+        <f>'data'!$B$8</f>
       </c>
     </row>
     <row r="7">
       <c r="F7" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G7" s="24"/>
       <c r="N7" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O7" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O7" s="24"/>
     </row>
     <row r="8">
       <c r="F8" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G8" s="24"/>
       <c r="N8" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O8" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O8" s="24"/>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="I11" s="27" t="s">
+      <c r="A11" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="27"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="I11" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
     </row>
     <row r="12">
       <c r="A12" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D12" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I12" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="L12" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I12" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L12" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O12" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="str">
-        <f>'data'!$B$9</f>
+        <f>'data'!$B$10</f>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -3142,10 +3193,10 @@
       <c r="E13" s="28"/>
       <c r="F13" s="28"/>
       <c r="G13" s="28" t="str">
-        <f>'data'!$B$11</f>
+        <f>'data'!$B$12</f>
       </c>
       <c r="I13" s="28" t="str">
-        <f>'data'!$B$12</f>
+        <f>'data'!$B$13</f>
       </c>
       <c r="J13" s="28"/>
       <c r="K13" s="28"/>
@@ -3153,72 +3204,72 @@
       <c r="M13" s="28"/>
       <c r="N13" s="28"/>
       <c r="O13" s="28" t="str">
-        <f>'data'!$B$13</f>
+        <f>'data'!$B$14</f>
       </c>
     </row>
     <row r="15">
       <c r="F15" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G15" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G15" s="24"/>
       <c r="N15" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O15" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O15" s="24"/>
     </row>
     <row r="16">
       <c r="F16" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G16" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G16" s="24"/>
       <c r="N16" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O16" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O16" s="24"/>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="I19" s="27" t="s">
+      <c r="A19" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-      <c r="O19" s="27"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="I19" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="20"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="20"/>
     </row>
     <row r="20">
       <c r="A20" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D20" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I20" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="30" t="s">
+      <c r="L20" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I20" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L20" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O20" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="str">
-        <f>'data'!$B$15</f>
+        <f>'data'!$B$16</f>
       </c>
       <c r="B21" s="28"/>
       <c r="C21" s="28"/>
@@ -3226,10 +3277,10 @@
       <c r="E21" s="28"/>
       <c r="F21" s="28"/>
       <c r="G21" s="28" t="str">
-        <f>'data'!$B$16</f>
+        <f>'data'!$B$17</f>
       </c>
       <c r="I21" s="28" t="str">
-        <f>'data'!$B$18</f>
+        <f>'data'!$B$19</f>
       </c>
       <c r="J21" s="28"/>
       <c r="K21" s="28"/>
@@ -3237,72 +3288,72 @@
       <c r="M21" s="28"/>
       <c r="N21" s="28"/>
       <c r="O21" s="28" t="str">
-        <f>'data'!$B$19</f>
+        <f>'data'!$B$20</f>
       </c>
     </row>
     <row r="23">
       <c r="F23" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G23" s="24"/>
       <c r="N23" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O23" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O23" s="24"/>
     </row>
     <row r="24">
       <c r="F24" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G24" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G24" s="24"/>
       <c r="N24" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O24" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O24" s="24"/>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="I27" s="27" t="s">
+      <c r="A27" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="27"/>
-      <c r="N27" s="27"/>
-      <c r="O27" s="27"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="I27" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
+      <c r="L27" s="20"/>
+      <c r="M27" s="20"/>
+      <c r="N27" s="20"/>
+      <c r="O27" s="20"/>
     </row>
     <row r="28">
       <c r="A28" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D28" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G28" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I28" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G28" s="30" t="s">
+      <c r="L28" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I28" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L28" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O28" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="str">
-        <f>'data'!$B$21</f>
+        <f>'data'!$B$22</f>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28"/>
@@ -3310,10 +3361,10 @@
       <c r="E29" s="28"/>
       <c r="F29" s="28"/>
       <c r="G29" s="28" t="str">
-        <f>'data'!$B$22</f>
+        <f>'data'!$B$23</f>
       </c>
       <c r="I29" s="28" t="str">
-        <f>'data'!$B$24</f>
+        <f>'data'!$B$25</f>
       </c>
       <c r="J29" s="28"/>
       <c r="K29" s="28"/>
@@ -3321,91 +3372,91 @@
       <c r="M29" s="28"/>
       <c r="N29" s="28"/>
       <c r="O29" s="28" t="str">
-        <f>'data'!$B$25</f>
+        <f>'data'!$B$26</f>
       </c>
     </row>
     <row r="31">
       <c r="F31" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G31" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G31" s="24"/>
       <c r="N31" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O31" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O31" s="24"/>
     </row>
     <row r="32">
       <c r="F32" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G32" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G32" s="24"/>
       <c r="N32" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O32" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O32" s="24"/>
     </row>
     <row r="40">
-      <c r="A40" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="27"/>
-      <c r="M40" s="27"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="27"/>
+      <c r="A40" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="20"/>
+      <c r="N40" s="20"/>
+      <c r="O40" s="20"/>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="B42" s="27"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="I42" s="27" t="s">
+      <c r="A42" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="J42" s="27"/>
-      <c r="K42" s="27"/>
-      <c r="L42" s="27"/>
-      <c r="M42" s="27"/>
-      <c r="N42" s="27"/>
-      <c r="O42" s="27"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="20"/>
+      <c r="I42" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="J42" s="20"/>
+      <c r="K42" s="20"/>
+      <c r="L42" s="20"/>
+      <c r="M42" s="20"/>
+      <c r="N42" s="20"/>
+      <c r="O42" s="20"/>
     </row>
     <row r="43">
       <c r="A43" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D43" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G43" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I43" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G43" s="30" t="s">
+      <c r="L43" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I43" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L43" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O43" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="28" t="str">
-        <f>'data'!$B$20</f>
+        <f>'data'!$B$21</f>
       </c>
       <c r="B44" s="28"/>
       <c r="C44" s="28"/>
@@ -3416,7 +3467,7 @@
         <f>CONCATENATE("M 1 ",'Elimination Matches'!G7)</f>
       </c>
       <c r="I44" s="28" t="str">
-        <f>'data'!$B$5</f>
+        <f>'data'!$B$6</f>
       </c>
       <c r="J44" s="28"/>
       <c r="K44" s="28"/>
@@ -3429,67 +3480,67 @@
     </row>
     <row r="46">
       <c r="F46" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G46" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G46" s="24"/>
       <c r="N46" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O46" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O46" s="24"/>
     </row>
     <row r="47">
       <c r="F47" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G47" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G47" s="24"/>
       <c r="N47" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O47" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O47" s="24"/>
     </row>
     <row r="50">
-      <c r="A50" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="B50" s="27"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="27"/>
-      <c r="E50" s="27"/>
-      <c r="F50" s="27"/>
-      <c r="G50" s="27"/>
-      <c r="I50" s="27" t="s">
+      <c r="A50" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="J50" s="27"/>
-      <c r="K50" s="27"/>
-      <c r="L50" s="27"/>
-      <c r="M50" s="27"/>
-      <c r="N50" s="27"/>
-      <c r="O50" s="27"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="20"/>
+      <c r="F50" s="20"/>
+      <c r="G50" s="20"/>
+      <c r="I50" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="J50" s="20"/>
+      <c r="K50" s="20"/>
+      <c r="L50" s="20"/>
+      <c r="M50" s="20"/>
+      <c r="N50" s="20"/>
+      <c r="O50" s="20"/>
     </row>
     <row r="51">
       <c r="A51" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D51" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G51" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I51" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G51" s="30" t="s">
+      <c r="L51" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I51" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L51" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O51" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="28" t="str">
-        <f>'data'!$B$8</f>
+        <f>'data'!$B$9</f>
       </c>
       <c r="B52" s="28"/>
       <c r="C52" s="28"/>
@@ -3500,7 +3551,7 @@
         <f>CONCATENATE("M 3 ",'Elimination Matches'!G15)</f>
       </c>
       <c r="I52" s="28" t="str">
-        <f>'data'!$B$11</f>
+        <f>'data'!$B$12</f>
       </c>
       <c r="J52" s="28"/>
       <c r="K52" s="28"/>
@@ -3513,67 +3564,67 @@
     </row>
     <row r="54">
       <c r="F54" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G54" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G54" s="24"/>
       <c r="N54" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O54" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O54" s="24"/>
     </row>
     <row r="55">
       <c r="F55" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G55" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G55" s="24"/>
       <c r="N55" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O55" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O55" s="24"/>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="B58" s="27"/>
-      <c r="C58" s="27"/>
-      <c r="D58" s="27"/>
-      <c r="E58" s="27"/>
-      <c r="F58" s="27"/>
-      <c r="G58" s="27"/>
-      <c r="I58" s="27" t="s">
+      <c r="A58" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="J58" s="27"/>
-      <c r="K58" s="27"/>
-      <c r="L58" s="27"/>
-      <c r="M58" s="27"/>
-      <c r="N58" s="27"/>
-      <c r="O58" s="27"/>
+      <c r="B58" s="20"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="20"/>
+      <c r="E58" s="20"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="20"/>
+      <c r="I58" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="J58" s="20"/>
+      <c r="K58" s="20"/>
+      <c r="L58" s="20"/>
+      <c r="M58" s="20"/>
+      <c r="N58" s="20"/>
+      <c r="O58" s="20"/>
     </row>
     <row r="59">
       <c r="A59" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D59" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G59" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I59" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G59" s="30" t="s">
+      <c r="L59" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I59" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L59" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O59" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="28" t="str">
-        <f>'data'!$B$14</f>
+        <f>'data'!$B$15</f>
       </c>
       <c r="B60" s="28"/>
       <c r="C60" s="28"/>
@@ -3584,7 +3635,7 @@
         <f>CONCATENATE("M 5 ",'Elimination Matches'!G23)</f>
       </c>
       <c r="I60" s="28" t="str">
-        <f>'data'!$B$17</f>
+        <f>'data'!$B$18</f>
       </c>
       <c r="J60" s="28"/>
       <c r="K60" s="28"/>
@@ -3597,67 +3648,67 @@
     </row>
     <row r="62">
       <c r="F62" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G62" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G62" s="24"/>
       <c r="N62" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O62" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O62" s="24"/>
     </row>
     <row r="63">
       <c r="F63" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G63" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G63" s="24"/>
       <c r="N63" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O63" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O63" s="24"/>
     </row>
     <row r="66">
-      <c r="A66" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="B66" s="27"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="27"/>
-      <c r="E66" s="27"/>
-      <c r="F66" s="27"/>
-      <c r="G66" s="27"/>
-      <c r="I66" s="27" t="s">
+      <c r="A66" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="J66" s="27"/>
-      <c r="K66" s="27"/>
-      <c r="L66" s="27"/>
-      <c r="M66" s="27"/>
-      <c r="N66" s="27"/>
-      <c r="O66" s="27"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="I66" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="J66" s="20"/>
+      <c r="K66" s="20"/>
+      <c r="L66" s="20"/>
+      <c r="M66" s="20"/>
+      <c r="N66" s="20"/>
+      <c r="O66" s="20"/>
     </row>
     <row r="67">
       <c r="A67" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D67" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G67" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I67" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G67" s="30" t="s">
+      <c r="L67" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I67" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L67" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O67" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="28" t="str">
-        <f>'data'!$B$20</f>
+        <f>'data'!$B$21</f>
       </c>
       <c r="B68" s="28"/>
       <c r="C68" s="28"/>
@@ -3668,7 +3719,7 @@
         <f>CONCATENATE("M 7 ",'Elimination Matches'!G31)</f>
       </c>
       <c r="I68" s="28" t="str">
-        <f>'data'!$B$23</f>
+        <f>'data'!$B$24</f>
       </c>
       <c r="J68" s="28"/>
       <c r="K68" s="28"/>
@@ -3681,81 +3732,81 @@
     </row>
     <row r="70">
       <c r="F70" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G70" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G70" s="24"/>
       <c r="N70" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O70" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O70" s="24"/>
     </row>
     <row r="71">
       <c r="F71" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G71" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G71" s="24"/>
       <c r="N71" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O71" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O71" s="24"/>
     </row>
     <row r="79">
-      <c r="A79" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="B79" s="27"/>
-      <c r="C79" s="27"/>
-      <c r="D79" s="27"/>
-      <c r="E79" s="27"/>
-      <c r="F79" s="27"/>
-      <c r="G79" s="27"/>
-      <c r="H79" s="27"/>
-      <c r="I79" s="27"/>
-      <c r="J79" s="27"/>
-      <c r="K79" s="27"/>
-      <c r="L79" s="27"/>
-      <c r="M79" s="27"/>
-      <c r="N79" s="27"/>
-      <c r="O79" s="27"/>
+      <c r="A79" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B79" s="20"/>
+      <c r="C79" s="20"/>
+      <c r="D79" s="20"/>
+      <c r="E79" s="20"/>
+      <c r="F79" s="20"/>
+      <c r="G79" s="20"/>
+      <c r="H79" s="20"/>
+      <c r="I79" s="20"/>
+      <c r="J79" s="20"/>
+      <c r="K79" s="20"/>
+      <c r="L79" s="20"/>
+      <c r="M79" s="20"/>
+      <c r="N79" s="20"/>
+      <c r="O79" s="20"/>
     </row>
     <row r="81">
-      <c r="A81" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="B81" s="27"/>
-      <c r="C81" s="27"/>
-      <c r="D81" s="27"/>
-      <c r="E81" s="27"/>
-      <c r="F81" s="27"/>
-      <c r="G81" s="27"/>
-      <c r="I81" s="27" t="s">
+      <c r="A81" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="J81" s="27"/>
-      <c r="K81" s="27"/>
-      <c r="L81" s="27"/>
-      <c r="M81" s="27"/>
-      <c r="N81" s="27"/>
-      <c r="O81" s="27"/>
+      <c r="B81" s="20"/>
+      <c r="C81" s="20"/>
+      <c r="D81" s="20"/>
+      <c r="E81" s="20"/>
+      <c r="F81" s="20"/>
+      <c r="G81" s="20"/>
+      <c r="I81" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="J81" s="20"/>
+      <c r="K81" s="20"/>
+      <c r="L81" s="20"/>
+      <c r="M81" s="20"/>
+      <c r="N81" s="20"/>
+      <c r="O81" s="20"/>
     </row>
     <row r="82">
       <c r="A82" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D82" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G82" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I82" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G82" s="30" t="s">
+      <c r="L82" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I82" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L82" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O82" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="83">
@@ -3784,62 +3835,62 @@
     </row>
     <row r="85">
       <c r="F85" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G85" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G85" s="24"/>
       <c r="N85" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O85" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O85" s="24"/>
     </row>
     <row r="86">
       <c r="F86" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G86" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G86" s="24"/>
       <c r="N86" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O86" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O86" s="24"/>
     </row>
     <row r="89">
-      <c r="A89" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="B89" s="27"/>
-      <c r="C89" s="27"/>
-      <c r="D89" s="27"/>
-      <c r="E89" s="27"/>
-      <c r="F89" s="27"/>
-      <c r="G89" s="27"/>
-      <c r="I89" s="27" t="s">
+      <c r="A89" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="J89" s="27"/>
-      <c r="K89" s="27"/>
-      <c r="L89" s="27"/>
-      <c r="M89" s="27"/>
-      <c r="N89" s="27"/>
-      <c r="O89" s="27"/>
+      <c r="B89" s="20"/>
+      <c r="C89" s="20"/>
+      <c r="D89" s="20"/>
+      <c r="E89" s="20"/>
+      <c r="F89" s="20"/>
+      <c r="G89" s="20"/>
+      <c r="I89" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="J89" s="20"/>
+      <c r="K89" s="20"/>
+      <c r="L89" s="20"/>
+      <c r="M89" s="20"/>
+      <c r="N89" s="20"/>
+      <c r="O89" s="20"/>
     </row>
     <row r="90">
       <c r="A90" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D90" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G90" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I90" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G90" s="30" t="s">
+      <c r="L90" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I90" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L90" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O90" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="91">
@@ -3868,81 +3919,81 @@
     </row>
     <row r="93">
       <c r="F93" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G93" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G93" s="24"/>
       <c r="N93" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O93" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O93" s="24"/>
     </row>
     <row r="94">
       <c r="F94" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G94" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G94" s="24"/>
       <c r="N94" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O94" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O94" s="24"/>
     </row>
     <row r="102">
-      <c r="A102" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B102" s="27"/>
-      <c r="C102" s="27"/>
-      <c r="D102" s="27"/>
-      <c r="E102" s="27"/>
-      <c r="F102" s="27"/>
-      <c r="G102" s="27"/>
-      <c r="H102" s="27"/>
-      <c r="I102" s="27"/>
-      <c r="J102" s="27"/>
-      <c r="K102" s="27"/>
-      <c r="L102" s="27"/>
-      <c r="M102" s="27"/>
-      <c r="N102" s="27"/>
-      <c r="O102" s="27"/>
+      <c r="A102" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="B102" s="20"/>
+      <c r="C102" s="20"/>
+      <c r="D102" s="20"/>
+      <c r="E102" s="20"/>
+      <c r="F102" s="20"/>
+      <c r="G102" s="20"/>
+      <c r="H102" s="20"/>
+      <c r="I102" s="20"/>
+      <c r="J102" s="20"/>
+      <c r="K102" s="20"/>
+      <c r="L102" s="20"/>
+      <c r="M102" s="20"/>
+      <c r="N102" s="20"/>
+      <c r="O102" s="20"/>
     </row>
     <row r="104">
-      <c r="A104" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="B104" s="27"/>
-      <c r="C104" s="27"/>
-      <c r="D104" s="27"/>
-      <c r="E104" s="27"/>
-      <c r="F104" s="27"/>
-      <c r="G104" s="27"/>
-      <c r="I104" s="27" t="s">
+      <c r="A104" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="J104" s="27"/>
-      <c r="K104" s="27"/>
-      <c r="L104" s="27"/>
-      <c r="M104" s="27"/>
-      <c r="N104" s="27"/>
-      <c r="O104" s="27"/>
+      <c r="B104" s="20"/>
+      <c r="C104" s="20"/>
+      <c r="D104" s="20"/>
+      <c r="E104" s="20"/>
+      <c r="F104" s="20"/>
+      <c r="G104" s="20"/>
+      <c r="I104" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="J104" s="20"/>
+      <c r="K104" s="20"/>
+      <c r="L104" s="20"/>
+      <c r="M104" s="20"/>
+      <c r="N104" s="20"/>
+      <c r="O104" s="20"/>
     </row>
     <row r="105">
       <c r="A105" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D105" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="G105" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I105" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="G105" s="30" t="s">
+      <c r="L105" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="I105" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="L105" s="28" t="s">
-        <v>86</v>
-      </c>
       <c r="O105" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="106">
@@ -3971,63 +4022,63 @@
     </row>
     <row r="108">
       <c r="F108" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G108" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G108" s="24"/>
       <c r="N108" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="O108" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="O108" s="24"/>
     </row>
     <row r="109">
       <c r="F109" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G109" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G109" s="24"/>
       <c r="N109" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="O109" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="O109" s="24"/>
     </row>
     <row r="117">
-      <c r="A117" s="27" t="s">
-        <v>114</v>
-      </c>
-      <c r="B117" s="27"/>
-      <c r="C117" s="27"/>
-      <c r="D117" s="27"/>
-      <c r="E117" s="27"/>
-      <c r="F117" s="27"/>
-      <c r="G117" s="27"/>
-      <c r="H117" s="27"/>
-      <c r="I117" s="27"/>
-      <c r="J117" s="27"/>
-      <c r="K117" s="27"/>
-      <c r="L117" s="27"/>
-      <c r="M117" s="27"/>
-      <c r="N117" s="27"/>
-      <c r="O117" s="27"/>
+      <c r="A117" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="B117" s="20"/>
+      <c r="C117" s="20"/>
+      <c r="D117" s="20"/>
+      <c r="E117" s="20"/>
+      <c r="F117" s="20"/>
+      <c r="G117" s="20"/>
+      <c r="H117" s="20"/>
+      <c r="I117" s="20"/>
+      <c r="J117" s="20"/>
+      <c r="K117" s="20"/>
+      <c r="L117" s="20"/>
+      <c r="M117" s="20"/>
+      <c r="N117" s="20"/>
+      <c r="O117" s="20"/>
     </row>
     <row r="119">
-      <c r="A119" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="B119" s="27"/>
-      <c r="C119" s="27"/>
-      <c r="D119" s="27"/>
-      <c r="E119" s="27"/>
-      <c r="F119" s="27"/>
-      <c r="G119" s="27"/>
+      <c r="A119" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="B119" s="20"/>
+      <c r="C119" s="20"/>
+      <c r="D119" s="20"/>
+      <c r="E119" s="20"/>
+      <c r="F119" s="20"/>
+      <c r="G119" s="20"/>
     </row>
     <row r="120">
       <c r="A120" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D120" s="28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G120" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="121">
@@ -4045,15 +4096,15 @@
     </row>
     <row r="123">
       <c r="F123" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G123" s="23"/>
+        <v>89</v>
+      </c>
+      <c r="G123" s="24"/>
     </row>
     <row r="124">
       <c r="F124" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G124" s="23"/>
+        <v>90</v>
+      </c>
+      <c r="G124" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="28">
@@ -4104,292 +4155,292 @@
   </cols>
   <sheetData>
     <row r="1" ht="110" customHeight="true">
-      <c r="A1" s="25">
+      <c r="A1" s="26">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="str">
-        <f>data!D2</f>
+      <c r="B1" s="27" t="str">
+        <f>data!D3</f>
       </c>
     </row>
     <row r="2" ht="115" customHeight="true">
-      <c r="A2" s="25"/>
-      <c r="B2" s="26"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="27"/>
     </row>
     <row r="3" ht="110" customHeight="true">
-      <c r="A3" s="25">
+      <c r="A3" s="26">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="str">
-        <f>data!D3</f>
+      <c r="B3" s="27" t="str">
+        <f>data!D4</f>
       </c>
     </row>
     <row r="4" ht="115" customHeight="true">
-      <c r="A4" s="25"/>
-      <c r="B4" s="26"/>
+      <c r="A4" s="26"/>
+      <c r="B4" s="27"/>
     </row>
     <row r="5" ht="110" customHeight="true">
-      <c r="A5" s="25">
+      <c r="A5" s="26">
         <v>2</v>
       </c>
-      <c r="B5" s="26" t="str">
-        <f>data!D4</f>
+      <c r="B5" s="27" t="str">
+        <f>data!D5</f>
       </c>
     </row>
     <row r="6" ht="115" customHeight="true">
-      <c r="A6" s="25"/>
-      <c r="B6" s="26"/>
+      <c r="A6" s="26"/>
+      <c r="B6" s="27"/>
     </row>
     <row r="7" ht="110" customHeight="true">
-      <c r="A7" s="25">
+      <c r="A7" s="26">
         <v>3</v>
       </c>
-      <c r="B7" s="26" t="str">
-        <f>data!D5</f>
+      <c r="B7" s="27" t="str">
+        <f>data!D6</f>
       </c>
     </row>
     <row r="8" ht="115" customHeight="true">
-      <c r="A8" s="25"/>
-      <c r="B8" s="26"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="27"/>
     </row>
     <row r="9" ht="110" customHeight="true">
-      <c r="A9" s="25">
+      <c r="A9" s="26">
         <v>4</v>
       </c>
-      <c r="B9" s="26" t="str">
-        <f>data!D6</f>
+      <c r="B9" s="27" t="str">
+        <f>data!D7</f>
       </c>
     </row>
     <row r="10" ht="115" customHeight="true">
-      <c r="A10" s="25"/>
-      <c r="B10" s="26"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="27"/>
     </row>
     <row r="11" ht="110" customHeight="true">
-      <c r="A11" s="25">
+      <c r="A11" s="26">
         <v>5</v>
       </c>
-      <c r="B11" s="26" t="str">
-        <f>data!D7</f>
+      <c r="B11" s="27" t="str">
+        <f>data!D8</f>
       </c>
     </row>
     <row r="12" ht="115" customHeight="true">
-      <c r="A12" s="25"/>
-      <c r="B12" s="26"/>
+      <c r="A12" s="26"/>
+      <c r="B12" s="27"/>
     </row>
     <row r="13" ht="110" customHeight="true">
-      <c r="A13" s="25">
+      <c r="A13" s="26">
         <v>6</v>
       </c>
-      <c r="B13" s="26" t="str">
-        <f>data!D8</f>
+      <c r="B13" s="27" t="str">
+        <f>data!D9</f>
       </c>
     </row>
     <row r="14" ht="115" customHeight="true">
-      <c r="A14" s="25"/>
-      <c r="B14" s="26"/>
+      <c r="A14" s="26"/>
+      <c r="B14" s="27"/>
     </row>
     <row r="15" ht="110" customHeight="true">
-      <c r="A15" s="25">
+      <c r="A15" s="26">
         <v>7</v>
       </c>
-      <c r="B15" s="26" t="str">
-        <f>data!D9</f>
+      <c r="B15" s="27" t="str">
+        <f>data!D10</f>
       </c>
     </row>
     <row r="16" ht="115" customHeight="true">
-      <c r="A16" s="25"/>
-      <c r="B16" s="26"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="27"/>
     </row>
     <row r="17" ht="110" customHeight="true">
-      <c r="A17" s="25">
+      <c r="A17" s="26">
         <v>8</v>
       </c>
-      <c r="B17" s="26" t="str">
-        <f>data!D10</f>
+      <c r="B17" s="27" t="str">
+        <f>data!D11</f>
       </c>
     </row>
     <row r="18" ht="115" customHeight="true">
-      <c r="A18" s="25"/>
-      <c r="B18" s="26"/>
+      <c r="A18" s="26"/>
+      <c r="B18" s="27"/>
     </row>
     <row r="19" ht="110" customHeight="true">
-      <c r="A19" s="25">
+      <c r="A19" s="26">
         <v>9</v>
       </c>
-      <c r="B19" s="26" t="str">
-        <f>data!D11</f>
+      <c r="B19" s="27" t="str">
+        <f>data!D12</f>
       </c>
     </row>
     <row r="20" ht="115" customHeight="true">
-      <c r="A20" s="25"/>
-      <c r="B20" s="26"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="27"/>
     </row>
     <row r="21" ht="110" customHeight="true">
-      <c r="A21" s="25">
+      <c r="A21" s="26">
         <v>10</v>
       </c>
-      <c r="B21" s="26" t="str">
-        <f>data!D12</f>
+      <c r="B21" s="27" t="str">
+        <f>data!D13</f>
       </c>
     </row>
     <row r="22" ht="115" customHeight="true">
-      <c r="A22" s="25"/>
-      <c r="B22" s="26"/>
+      <c r="A22" s="26"/>
+      <c r="B22" s="27"/>
     </row>
     <row r="23" ht="110" customHeight="true">
-      <c r="A23" s="25">
+      <c r="A23" s="26">
         <v>11</v>
       </c>
-      <c r="B23" s="26" t="str">
-        <f>data!D13</f>
+      <c r="B23" s="27" t="str">
+        <f>data!D14</f>
       </c>
     </row>
     <row r="24" ht="115" customHeight="true">
-      <c r="A24" s="25"/>
-      <c r="B24" s="26"/>
+      <c r="A24" s="26"/>
+      <c r="B24" s="27"/>
     </row>
     <row r="25" ht="110" customHeight="true">
-      <c r="A25" s="25">
+      <c r="A25" s="26">
         <v>12</v>
       </c>
-      <c r="B25" s="26" t="str">
-        <f>data!D14</f>
+      <c r="B25" s="27" t="str">
+        <f>data!D15</f>
       </c>
     </row>
     <row r="26" ht="115" customHeight="true">
-      <c r="A26" s="25"/>
-      <c r="B26" s="26"/>
+      <c r="A26" s="26"/>
+      <c r="B26" s="27"/>
     </row>
     <row r="27" ht="110" customHeight="true">
-      <c r="A27" s="25">
+      <c r="A27" s="26">
         <v>13</v>
       </c>
-      <c r="B27" s="26" t="str">
-        <f>data!D15</f>
+      <c r="B27" s="27" t="str">
+        <f>data!D16</f>
       </c>
     </row>
     <row r="28" ht="115" customHeight="true">
-      <c r="A28" s="25"/>
-      <c r="B28" s="26"/>
+      <c r="A28" s="26"/>
+      <c r="B28" s="27"/>
     </row>
     <row r="29" ht="110" customHeight="true">
-      <c r="A29" s="25">
+      <c r="A29" s="26">
         <v>14</v>
       </c>
-      <c r="B29" s="26" t="str">
-        <f>data!D16</f>
+      <c r="B29" s="27" t="str">
+        <f>data!D17</f>
       </c>
     </row>
     <row r="30" ht="115" customHeight="true">
-      <c r="A30" s="25"/>
-      <c r="B30" s="26"/>
+      <c r="A30" s="26"/>
+      <c r="B30" s="27"/>
     </row>
     <row r="31" ht="110" customHeight="true">
-      <c r="A31" s="25">
+      <c r="A31" s="26">
         <v>15</v>
       </c>
-      <c r="B31" s="26" t="str">
-        <f>data!D17</f>
+      <c r="B31" s="27" t="str">
+        <f>data!D18</f>
       </c>
     </row>
     <row r="32" ht="115" customHeight="true">
-      <c r="A32" s="25"/>
-      <c r="B32" s="26"/>
+      <c r="A32" s="26"/>
+      <c r="B32" s="27"/>
     </row>
     <row r="33" ht="110" customHeight="true">
-      <c r="A33" s="25">
+      <c r="A33" s="26">
         <v>16</v>
       </c>
-      <c r="B33" s="26" t="str">
-        <f>data!D18</f>
+      <c r="B33" s="27" t="str">
+        <f>data!D19</f>
       </c>
     </row>
     <row r="34" ht="115" customHeight="true">
-      <c r="A34" s="25"/>
-      <c r="B34" s="26"/>
+      <c r="A34" s="26"/>
+      <c r="B34" s="27"/>
     </row>
     <row r="35" ht="110" customHeight="true">
-      <c r="A35" s="25">
+      <c r="A35" s="26">
         <v>17</v>
       </c>
-      <c r="B35" s="26" t="str">
-        <f>data!D19</f>
+      <c r="B35" s="27" t="str">
+        <f>data!D20</f>
       </c>
     </row>
     <row r="36" ht="115" customHeight="true">
-      <c r="A36" s="25"/>
-      <c r="B36" s="26"/>
+      <c r="A36" s="26"/>
+      <c r="B36" s="27"/>
     </row>
     <row r="37" ht="110" customHeight="true">
-      <c r="A37" s="25">
+      <c r="A37" s="26">
         <v>18</v>
       </c>
-      <c r="B37" s="26" t="str">
-        <f>data!D20</f>
+      <c r="B37" s="27" t="str">
+        <f>data!D21</f>
       </c>
     </row>
     <row r="38" ht="115" customHeight="true">
-      <c r="A38" s="25"/>
-      <c r="B38" s="26"/>
+      <c r="A38" s="26"/>
+      <c r="B38" s="27"/>
     </row>
     <row r="39" ht="110" customHeight="true">
-      <c r="A39" s="25">
+      <c r="A39" s="26">
         <v>19</v>
       </c>
-      <c r="B39" s="26" t="str">
-        <f>data!D21</f>
+      <c r="B39" s="27" t="str">
+        <f>data!D22</f>
       </c>
     </row>
     <row r="40" ht="115" customHeight="true">
-      <c r="A40" s="25"/>
-      <c r="B40" s="26"/>
+      <c r="A40" s="26"/>
+      <c r="B40" s="27"/>
     </row>
     <row r="41" ht="110" customHeight="true">
-      <c r="A41" s="25">
+      <c r="A41" s="26">
         <v>20</v>
       </c>
-      <c r="B41" s="26" t="str">
-        <f>data!D22</f>
+      <c r="B41" s="27" t="str">
+        <f>data!D23</f>
       </c>
     </row>
     <row r="42" ht="115" customHeight="true">
-      <c r="A42" s="25"/>
-      <c r="B42" s="26"/>
+      <c r="A42" s="26"/>
+      <c r="B42" s="27"/>
     </row>
     <row r="43" ht="110" customHeight="true">
-      <c r="A43" s="25">
+      <c r="A43" s="26">
         <v>21</v>
       </c>
-      <c r="B43" s="26" t="str">
-        <f>data!D23</f>
+      <c r="B43" s="27" t="str">
+        <f>data!D24</f>
       </c>
     </row>
     <row r="44" ht="115" customHeight="true">
-      <c r="A44" s="25"/>
-      <c r="B44" s="26"/>
+      <c r="A44" s="26"/>
+      <c r="B44" s="27"/>
     </row>
     <row r="45" ht="110" customHeight="true">
-      <c r="A45" s="25">
+      <c r="A45" s="26">
         <v>22</v>
       </c>
-      <c r="B45" s="26" t="str">
-        <f>data!D24</f>
+      <c r="B45" s="27" t="str">
+        <f>data!D25</f>
       </c>
     </row>
     <row r="46" ht="115" customHeight="true">
-      <c r="A46" s="25"/>
-      <c r="B46" s="26"/>
+      <c r="A46" s="26"/>
+      <c r="B46" s="27"/>
     </row>
     <row r="47" ht="110" customHeight="true">
-      <c r="A47" s="25">
+      <c r="A47" s="26">
         <v>23</v>
       </c>
-      <c r="B47" s="26" t="str">
-        <f>data!D25</f>
+      <c r="B47" s="27" t="str">
+        <f>data!D26</f>
       </c>
     </row>
     <row r="48" ht="115" customHeight="true">
-      <c r="A48" s="25"/>
-      <c r="B48" s="26"/>
+      <c r="A48" s="26"/>
+      <c r="B48" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>

<commit_message>
docs: add project management documentation and refactor pool-to-court assignment logic for improved robustness.
</commit_message>
<xml_diff>
--- a/playoffs-example-medium.xlsx
+++ b/playoffs-example-medium.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
   <si>
     <t>Elimination Round 1</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>Title prefix:</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Number</t>
@@ -957,23 +960,25 @@
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:2" ht="12.75" customHeight="true">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="12.75" customHeight="true">
@@ -981,13 +986,13 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="12.75" customHeight="true">
@@ -995,13 +1000,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="12.75" customHeight="true">
@@ -1009,13 +1014,13 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="12.75" customHeight="true">
@@ -1023,13 +1028,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="12.75" customHeight="true">
@@ -1037,13 +1042,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="12.75" customHeight="true">
@@ -1051,13 +1056,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="12.75" customHeight="true">
@@ -1065,13 +1070,13 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="12.75" customHeight="true">
@@ -1079,13 +1084,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="12.75" customHeight="true">
@@ -1093,13 +1098,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="12.75" customHeight="true">
@@ -1107,13 +1112,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" t="s">
         <v>44</v>
-      </c>
-      <c r="D12" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="12.75" customHeight="true">
@@ -1121,13 +1126,13 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
         <v>45</v>
       </c>
-      <c r="C13" t="s">
-        <v>44</v>
-      </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="12.75" customHeight="true">
@@ -1135,13 +1140,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="12.75" customHeight="true">
@@ -1149,13 +1154,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="12.75" customHeight="true">
@@ -1163,13 +1168,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="12.75" customHeight="true">
@@ -1177,13 +1182,13 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="12.75" customHeight="true">
@@ -1191,13 +1196,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="12.75" customHeight="true">
@@ -1205,13 +1210,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="12.75" customHeight="true">
@@ -1219,13 +1224,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="12.75" customHeight="true">
@@ -1233,13 +1238,13 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="12.75" customHeight="true">
@@ -1247,13 +1252,13 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="12.75" customHeight="true">
@@ -1261,13 +1266,13 @@
         <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="12.75" customHeight="true">
@@ -1275,13 +1280,13 @@
         <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="12.75" customHeight="true">
@@ -1289,13 +1294,13 @@
         <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D25" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="12.75" customHeight="true">
@@ -1303,13 +1308,13 @@
         <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="12.75" customHeight="true">
@@ -2374,7 +2379,7 @@
     </row>
     <row r="6">
       <c r="E6" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -2388,7 +2393,7 @@
     </row>
     <row r="9">
       <c r="C9" s="25" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="23"/>
@@ -2405,7 +2410,7 @@
     </row>
     <row r="11">
       <c r="C11" s="25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D11" s="24"/>
       <c r="E11" s="21"/>
@@ -2423,7 +2428,7 @@
     </row>
     <row r="14">
       <c r="E14" s="25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I14" s="21"/>
       <c r="K14" s="21"/>
@@ -2444,7 +2449,7 @@
     </row>
     <row r="17">
       <c r="C17" s="25" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G17" s="21"/>
       <c r="K17" s="21"/>
@@ -2460,7 +2465,7 @@
     </row>
     <row r="19">
       <c r="C19" s="25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D19" s="24"/>
       <c r="E19" s="21"/>
@@ -2476,7 +2481,7 @@
     </row>
     <row r="22">
       <c r="E22" s="25" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K22" s="21"/>
     </row>
@@ -2493,7 +2498,7 @@
     </row>
     <row r="25">
       <c r="C25" s="25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G25" s="21"/>
       <c r="H25" s="23"/>
@@ -2512,7 +2517,7 @@
     </row>
     <row r="27">
       <c r="C27" s="25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="21"/>
@@ -2531,7 +2536,7 @@
     </row>
     <row r="30">
       <c r="E30" s="25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I30" s="21"/>
     </row>
@@ -2549,7 +2554,7 @@
     </row>
     <row r="33">
       <c r="C33" s="25" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G33" s="21"/>
     </row>
@@ -2563,7 +2568,7 @@
     </row>
     <row r="35">
       <c r="C35" s="25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D35" s="24"/>
       <c r="E35" s="21"/>
@@ -2611,7 +2616,7 @@
     </row>
     <row r="6">
       <c r="E6" s="25" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -2625,7 +2630,7 @@
     </row>
     <row r="9">
       <c r="C9" s="25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="23"/>
@@ -2642,7 +2647,7 @@
     </row>
     <row r="11">
       <c r="C11" s="25" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D11" s="24"/>
       <c r="E11" s="21"/>
@@ -2660,7 +2665,7 @@
     </row>
     <row r="14">
       <c r="E14" s="25" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I14" s="21"/>
       <c r="K14" s="21"/>
@@ -2681,7 +2686,7 @@
     </row>
     <row r="17">
       <c r="C17" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G17" s="21"/>
       <c r="K17" s="21"/>
@@ -2697,7 +2702,7 @@
     </row>
     <row r="19">
       <c r="C19" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D19" s="24"/>
       <c r="E19" s="21"/>
@@ -2713,7 +2718,7 @@
     </row>
     <row r="22">
       <c r="E22" s="25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K22" s="21"/>
     </row>
@@ -2730,7 +2735,7 @@
     </row>
     <row r="25">
       <c r="C25" s="25" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G25" s="21"/>
       <c r="H25" s="23"/>
@@ -2749,7 +2754,7 @@
     </row>
     <row r="27">
       <c r="C27" s="25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="21"/>
@@ -2768,7 +2773,7 @@
     </row>
     <row r="30">
       <c r="E30" s="25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I30" s="21"/>
     </row>
@@ -2786,7 +2791,7 @@
     </row>
     <row r="33">
       <c r="C33" s="25" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G33" s="21"/>
     </row>
@@ -2800,7 +2805,7 @@
     </row>
     <row r="35">
       <c r="C35" s="25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D35" s="24"/>
       <c r="E35" s="21"/>
@@ -3026,18 +3031,19 @@
   <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="7" width="34"/>
-    <col customWidth="true" max="3" min="2" style="7" width="3.83203125"/>
+    <col customWidth="true" max="1" min="1" style="7" width="30"/>
+    <col customWidth="true" max="3" min="2" style="7" width="5"/>
     <col customWidth="true" max="4" min="4" style="7" width="3"/>
-    <col customWidth="true" max="6" min="5" style="7" width="3.83203125"/>
-    <col customWidth="true" max="7" min="7" style="7" width="34"/>
-    <col customWidth="true" max="8" min="8" style="7" width="3.83203125"/>
-    <col customWidth="true" max="9" min="9" style="7" width="34"/>
-    <col customWidth="true" max="11" min="10" style="7" width="3.83203125"/>
+    <col customWidth="true" max="6" min="5" style="7" width="5"/>
+    <col customWidth="true" max="7" min="7" style="7" width="30"/>
+    <col customWidth="true" max="8" min="8" style="7" width="2"/>
+    <col customWidth="true" max="9" min="9" style="7" width="30"/>
+    <col customWidth="true" max="11" min="10" style="7" width="5"/>
     <col customWidth="true" max="12" min="12" style="7" width="3"/>
-    <col customWidth="true" max="14" min="13" style="7" width="3.83203125"/>
-    <col customWidth="true" max="15" min="15" style="7" width="34"/>
-    <col max="16384" min="16" style="7" width="10.83203125"/>
+    <col customWidth="true" max="14" min="13" style="7" width="5"/>
+    <col customWidth="true" max="15" min="15" style="7" width="30"/>
+    <col customWidth="true" max="16" min="16" style="7" width="2"/>
+    <col max="16384" min="17" style="7" width="10.83203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17" thickBot="true">
@@ -3061,7 +3067,7 @@
     </row>
     <row r="3">
       <c r="A3" s="20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" s="20"/>
       <c r="C3" s="20"/>
@@ -3070,7 +3076,7 @@
       <c r="F3" s="20"/>
       <c r="G3" s="20"/>
       <c r="I3" s="20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J3" s="20"/>
       <c r="K3" s="20"/>
@@ -3081,22 +3087,22 @@
     </row>
     <row r="4">
       <c r="A4" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D4" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I4" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="L4" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I4" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L4" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O4" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5">
@@ -3125,27 +3131,27 @@
     </row>
     <row r="7">
       <c r="F7" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G7" s="24"/>
       <c r="N7" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O7" s="24"/>
     </row>
     <row r="8">
       <c r="F8" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G8" s="24"/>
       <c r="N8" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O8" s="24"/>
     </row>
     <row r="11">
       <c r="A11" s="20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3154,7 +3160,7 @@
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
       <c r="I11" s="20" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J11" s="20"/>
       <c r="K11" s="20"/>
@@ -3165,22 +3171,22 @@
     </row>
     <row r="12">
       <c r="A12" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D12" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G12" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I12" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="L12" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I12" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L12" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O12" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13">
@@ -3209,27 +3215,27 @@
     </row>
     <row r="15">
       <c r="F15" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G15" s="24"/>
       <c r="N15" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O15" s="24"/>
     </row>
     <row r="16">
       <c r="F16" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G16" s="24"/>
       <c r="N16" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O16" s="24"/>
     </row>
     <row r="19">
       <c r="A19" s="20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -3238,7 +3244,7 @@
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
       <c r="I19" s="20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J19" s="20"/>
       <c r="K19" s="20"/>
@@ -3249,22 +3255,22 @@
     </row>
     <row r="20">
       <c r="A20" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D20" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G20" s="30" t="s">
+      <c r="L20" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I20" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L20" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O20" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21">
@@ -3293,27 +3299,27 @@
     </row>
     <row r="23">
       <c r="F23" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G23" s="24"/>
       <c r="N23" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O23" s="24"/>
     </row>
     <row r="24">
       <c r="F24" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G24" s="24"/>
       <c r="N24" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O24" s="24"/>
     </row>
     <row r="27">
       <c r="A27" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
@@ -3322,7 +3328,7 @@
       <c r="F27" s="20"/>
       <c r="G27" s="20"/>
       <c r="I27" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J27" s="20"/>
       <c r="K27" s="20"/>
@@ -3333,22 +3339,22 @@
     </row>
     <row r="28">
       <c r="A28" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D28" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G28" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I28" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G28" s="30" t="s">
+      <c r="L28" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I28" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L28" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O28" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29">
@@ -3377,27 +3383,27 @@
     </row>
     <row r="31">
       <c r="F31" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G31" s="24"/>
       <c r="N31" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O31" s="24"/>
     </row>
     <row r="32">
       <c r="F32" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G32" s="24"/>
       <c r="N32" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O32" s="24"/>
     </row>
     <row r="40">
       <c r="A40" s="20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B40" s="20"/>
       <c r="C40" s="20"/>
@@ -3416,7 +3422,7 @@
     </row>
     <row r="42">
       <c r="A42" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B42" s="20"/>
       <c r="C42" s="20"/>
@@ -3425,7 +3431,7 @@
       <c r="F42" s="20"/>
       <c r="G42" s="20"/>
       <c r="I42" s="20" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J42" s="20"/>
       <c r="K42" s="20"/>
@@ -3436,22 +3442,22 @@
     </row>
     <row r="43">
       <c r="A43" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D43" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G43" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I43" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G43" s="30" t="s">
+      <c r="L43" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I43" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L43" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O43" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="44">
@@ -3480,27 +3486,27 @@
     </row>
     <row r="46">
       <c r="F46" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G46" s="24"/>
       <c r="N46" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O46" s="24"/>
     </row>
     <row r="47">
       <c r="F47" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G47" s="24"/>
       <c r="N47" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O47" s="24"/>
     </row>
     <row r="50">
       <c r="A50" s="20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B50" s="20"/>
       <c r="C50" s="20"/>
@@ -3509,7 +3515,7 @@
       <c r="F50" s="20"/>
       <c r="G50" s="20"/>
       <c r="I50" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J50" s="20"/>
       <c r="K50" s="20"/>
@@ -3520,22 +3526,22 @@
     </row>
     <row r="51">
       <c r="A51" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D51" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G51" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I51" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G51" s="30" t="s">
+      <c r="L51" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I51" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L51" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O51" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="52">
@@ -3564,27 +3570,27 @@
     </row>
     <row r="54">
       <c r="F54" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G54" s="24"/>
       <c r="N54" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O54" s="24"/>
     </row>
     <row r="55">
       <c r="F55" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G55" s="24"/>
       <c r="N55" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O55" s="24"/>
     </row>
     <row r="58">
       <c r="A58" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B58" s="20"/>
       <c r="C58" s="20"/>
@@ -3593,7 +3599,7 @@
       <c r="F58" s="20"/>
       <c r="G58" s="20"/>
       <c r="I58" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J58" s="20"/>
       <c r="K58" s="20"/>
@@ -3604,22 +3610,22 @@
     </row>
     <row r="59">
       <c r="A59" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D59" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G59" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I59" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G59" s="30" t="s">
+      <c r="L59" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I59" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L59" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O59" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60">
@@ -3648,27 +3654,27 @@
     </row>
     <row r="62">
       <c r="F62" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G62" s="24"/>
       <c r="N62" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O62" s="24"/>
     </row>
     <row r="63">
       <c r="F63" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G63" s="24"/>
       <c r="N63" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O63" s="24"/>
     </row>
     <row r="66">
       <c r="A66" s="20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B66" s="20"/>
       <c r="C66" s="20"/>
@@ -3677,7 +3683,7 @@
       <c r="F66" s="20"/>
       <c r="G66" s="20"/>
       <c r="I66" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J66" s="20"/>
       <c r="K66" s="20"/>
@@ -3688,22 +3694,22 @@
     </row>
     <row r="67">
       <c r="A67" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D67" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G67" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I67" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G67" s="30" t="s">
+      <c r="L67" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I67" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L67" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O67" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="68">
@@ -3732,27 +3738,27 @@
     </row>
     <row r="70">
       <c r="F70" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G70" s="24"/>
       <c r="N70" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O70" s="24"/>
     </row>
     <row r="71">
       <c r="F71" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G71" s="24"/>
       <c r="N71" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O71" s="24"/>
     </row>
     <row r="79">
       <c r="A79" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B79" s="20"/>
       <c r="C79" s="20"/>
@@ -3771,7 +3777,7 @@
     </row>
     <row r="81">
       <c r="A81" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B81" s="20"/>
       <c r="C81" s="20"/>
@@ -3780,7 +3786,7 @@
       <c r="F81" s="20"/>
       <c r="G81" s="20"/>
       <c r="I81" s="20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J81" s="20"/>
       <c r="K81" s="20"/>
@@ -3791,22 +3797,22 @@
     </row>
     <row r="82">
       <c r="A82" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D82" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G82" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I82" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G82" s="30" t="s">
+      <c r="L82" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I82" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L82" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O82" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="83">
@@ -3835,27 +3841,27 @@
     </row>
     <row r="85">
       <c r="F85" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G85" s="24"/>
       <c r="N85" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O85" s="24"/>
     </row>
     <row r="86">
       <c r="F86" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G86" s="24"/>
       <c r="N86" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O86" s="24"/>
     </row>
     <row r="89">
       <c r="A89" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B89" s="20"/>
       <c r="C89" s="20"/>
@@ -3864,7 +3870,7 @@
       <c r="F89" s="20"/>
       <c r="G89" s="20"/>
       <c r="I89" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J89" s="20"/>
       <c r="K89" s="20"/>
@@ -3875,22 +3881,22 @@
     </row>
     <row r="90">
       <c r="A90" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D90" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G90" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I90" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G90" s="30" t="s">
+      <c r="L90" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I90" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L90" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O90" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="91">
@@ -3919,27 +3925,27 @@
     </row>
     <row r="93">
       <c r="F93" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G93" s="24"/>
       <c r="N93" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O93" s="24"/>
     </row>
     <row r="94">
       <c r="F94" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G94" s="24"/>
       <c r="N94" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O94" s="24"/>
     </row>
     <row r="102">
       <c r="A102" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B102" s="20"/>
       <c r="C102" s="20"/>
@@ -3958,7 +3964,7 @@
     </row>
     <row r="104">
       <c r="A104" s="20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B104" s="20"/>
       <c r="C104" s="20"/>
@@ -3967,7 +3973,7 @@
       <c r="F104" s="20"/>
       <c r="G104" s="20"/>
       <c r="I104" s="20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J104" s="20"/>
       <c r="K104" s="20"/>
@@ -3978,22 +3984,22 @@
     </row>
     <row r="105">
       <c r="A105" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D105" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="G105" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I105" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G105" s="30" t="s">
+      <c r="L105" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="I105" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="L105" s="28" t="s">
-        <v>87</v>
-      </c>
       <c r="O105" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="106">
@@ -4022,27 +4028,27 @@
     </row>
     <row r="108">
       <c r="F108" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G108" s="24"/>
       <c r="N108" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O108" s="24"/>
     </row>
     <row r="109">
       <c r="F109" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G109" s="24"/>
       <c r="N109" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O109" s="24"/>
     </row>
     <row r="117">
       <c r="A117" s="20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B117" s="20"/>
       <c r="C117" s="20"/>
@@ -4061,7 +4067,7 @@
     </row>
     <row r="119">
       <c r="A119" s="20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B119" s="20"/>
       <c r="C119" s="20"/>
@@ -4072,13 +4078,13 @@
     </row>
     <row r="120">
       <c r="A120" s="29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D120" s="28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G120" s="30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="121">
@@ -4096,13 +4102,13 @@
     </row>
     <row r="123">
       <c r="F123" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G123" s="24"/>
     </row>
     <row r="124">
       <c r="F124" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G124" s="24"/>
     </row>

</xml_diff>

<commit_message>
refactor: adjust Excel row calculations and update test expectations for match layouts
</commit_message>
<xml_diff>
--- a/playoffs-example-medium.xlsx
+++ b/playoffs-example-medium.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="26060" windowHeight="21580" activeTab="1"/>
+    <workbookView xWindow="34720" yWindow="1400" windowWidth="38080" windowHeight="20800" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
   </sheets>
   <definedNames>
     <definedName localSheetId="3" name="_xlnm.Print_Area">'Names to Print'!$A$1:$B$48</definedName>
+    <definedName localSheetId="2" name="_xlnm.Print_Area">'Elimination Matches'!$A$1:$O$122</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,10 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
-  <si>
-    <t>Elimination Round 1</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
   <si>
     <t>Tournament Pools</t>
   </si>
@@ -303,7 +301,13 @@
     <t>YGRITTE</t>
   </si>
   <si>
-    <t>Match 1</t>
+    <t>Shiaijo A</t>
+  </si>
+  <si>
+    <t>Shiaijo B</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 1</t>
   </si>
   <si>
     <t>White</t>
@@ -321,82 +325,91 @@
     <t>2.</t>
   </si>
   <si>
-    <t>Match 2</t>
-  </si>
-  <si>
-    <t>Match 3</t>
-  </si>
-  <si>
-    <t>Match 4</t>
-  </si>
-  <si>
-    <t>Match 5</t>
-  </si>
-  <si>
-    <t>Match 6</t>
-  </si>
-  <si>
-    <t>Match 7</t>
-  </si>
-  <si>
-    <t>Match 8</t>
-  </si>
-  <si>
-    <t>Elimination Round 2</t>
-  </si>
-  <si>
-    <t>Match 9</t>
-  </si>
-  <si>
-    <t>Match 10</t>
-  </si>
-  <si>
-    <t>Match 11</t>
-  </si>
-  <si>
-    <t>Match 12</t>
-  </si>
-  <si>
-    <t>Match 13</t>
-  </si>
-  <si>
-    <t>Match 14</t>
-  </si>
-  <si>
-    <t>Match 15</t>
-  </si>
-  <si>
-    <t>Match 16</t>
-  </si>
-  <si>
-    <t>Elimination Round 3</t>
-  </si>
-  <si>
-    <t>Match 17</t>
-  </si>
-  <si>
-    <t>Match 18</t>
-  </si>
-  <si>
-    <t>Match 19</t>
-  </si>
-  <si>
-    <t>Match 20</t>
-  </si>
-  <si>
-    <t>Elimination Round 4</t>
-  </si>
-  <si>
-    <t>Match 21</t>
-  </si>
-  <si>
-    <t>Match 22</t>
-  </si>
-  <si>
-    <t>Elimination Round 5</t>
-  </si>
-  <si>
-    <t>Match 0</t>
+    <t>Round 1 - Match 5</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 2</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 6</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 3</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 7</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 4</t>
+  </si>
+  <si>
+    <t>Round 1 - Match 8</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 9</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 13</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 10</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 14</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 11</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 15</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 12</t>
+  </si>
+  <si>
+    <t>Round 2 - Match 16</t>
+  </si>
+  <si>
+    <t>Round 3 - Match 17</t>
+  </si>
+  <si>
+    <t>Round 3 - Match 19</t>
+  </si>
+  <si>
+    <t>Round 3 - Match 18</t>
+  </si>
+  <si>
+    <t>Round 3 - Match 20</t>
+  </si>
+  <si>
+    <t>Round 4 - Match 21</t>
+  </si>
+  <si>
+    <t>Round 4 - Match 22</t>
+  </si>
+  <si>
+    <t>Round 5 - Match 0</t>
+  </si>
+  <si>
+    <t>Tournament Summary</t>
+  </si>
+  <si>
+    <t>Total Pool Time</t>
+  </si>
+  <si>
+    <t>Total Elimination Time</t>
+  </si>
+  <si>
+    <t>Grand Total (Sequential)</t>
+  </si>
+  <si>
+    <t>Grand Total (Parallel across Courts)</t>
+  </si>
+  <si>
+    <t>Start Time:</t>
+  </si>
+  <si>
+    <t>Estimated Finish Time</t>
   </si>
 </sst>
 </file>
@@ -539,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -559,43 +572,6 @@
       </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -654,7 +630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -692,46 +668,41 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -958,27 +929,27 @@
   <sheetData>
     <row r="1" spans="1:2" ht="12.75" customHeight="true">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="12.75" customHeight="true">
       <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="12.75" customHeight="true">
@@ -986,13 +957,13 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="12.75" customHeight="true">
@@ -1000,13 +971,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="12.75" customHeight="true">
@@ -1014,13 +985,13 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="12.75" customHeight="true">
@@ -1028,13 +999,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>28</v>
-      </c>
-      <c r="D6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="12.75" customHeight="true">
@@ -1042,13 +1013,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="12.75" customHeight="true">
@@ -1056,13 +1027,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="12.75" customHeight="true">
@@ -1070,13 +1041,13 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
         <v>36</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>37</v>
-      </c>
-      <c r="D9" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="12.75" customHeight="true">
@@ -1084,13 +1055,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
         <v>39</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>40</v>
-      </c>
-      <c r="D10" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="12.75" customHeight="true">
@@ -1098,13 +1069,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>43</v>
-      </c>
-      <c r="D11" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="12.75" customHeight="true">
@@ -1112,13 +1083,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="12.75" customHeight="true">
@@ -1126,13 +1097,13 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
         <v>46</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="12.75" customHeight="true">
@@ -1140,13 +1111,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
         <v>48</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>49</v>
-      </c>
-      <c r="D14" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="12.75" customHeight="true">
@@ -1154,13 +1125,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
         <v>51</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>52</v>
-      </c>
-      <c r="D15" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="12.75" customHeight="true">
@@ -1168,13 +1139,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
         <v>54</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>55</v>
-      </c>
-      <c r="D16" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="12.75" customHeight="true">
@@ -1182,13 +1153,13 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
         <v>57</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>58</v>
-      </c>
-      <c r="D17" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="12.75" customHeight="true">
@@ -1196,13 +1167,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
         <v>60</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>61</v>
-      </c>
-      <c r="D18" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="12.75" customHeight="true">
@@ -1210,13 +1181,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" t="s">
         <v>63</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>64</v>
-      </c>
-      <c r="D19" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="12.75" customHeight="true">
@@ -1224,13 +1195,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
         <v>66</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>67</v>
-      </c>
-      <c r="D20" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="12.75" customHeight="true">
@@ -1238,13 +1209,13 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
         <v>69</v>
       </c>
-      <c r="C21" t="s">
-        <v>70</v>
-      </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="12.75" customHeight="true">
@@ -1252,13 +1223,13 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" t="s">
         <v>71</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>72</v>
-      </c>
-      <c r="D22" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="12.75" customHeight="true">
@@ -1266,13 +1237,13 @@
         <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" t="s">
         <v>74</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>75</v>
-      </c>
-      <c r="D23" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="12.75" customHeight="true">
@@ -1280,13 +1251,13 @@
         <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" t="s">
         <v>77</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>78</v>
-      </c>
-      <c r="D24" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="12.75" customHeight="true">
@@ -1294,13 +1265,13 @@
         <v>22</v>
       </c>
       <c r="B25" t="s">
+        <v>79</v>
+      </c>
+      <c r="C25" t="s">
         <v>80</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>81</v>
-      </c>
-      <c r="D25" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="12.75" customHeight="true">
@@ -1308,13 +1279,13 @@
         <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" t="s">
         <v>83</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>84</v>
-      </c>
-      <c r="D26" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="12.75" customHeight="true">
@@ -2358,220 +2329,220 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="str">
+      <c r="A1" s="18" t="str">
         <f>IF(data!$B$1="","Shiaijo A",data!$B$1&amp;" - Shiaijo A")</f>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
     </row>
     <row r="6">
-      <c r="E6" s="25" t="s">
-        <v>20</v>
+      <c r="E6" s="23" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7">
-      <c r="F7" s="23"/>
-      <c r="G7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="19"/>
     </row>
     <row r="8">
-      <c r="G8" s="22">
+      <c r="G8" s="20">
         <v>9</v>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="21"/>
+      <c r="C9" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="19"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10">
-      <c r="D10" s="23"/>
-      <c r="E10" s="22">
+      <c r="D10" s="21"/>
+      <c r="E10" s="20">
         <v>1</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="21"/>
-      <c r="I10" s="21"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11">
-      <c r="C11" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="21"/>
-      <c r="I11" s="21"/>
+      <c r="C11" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="22"/>
+      <c r="E11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12">
-      <c r="I12" s="22">
+      <c r="I12" s="20">
         <v>17</v>
       </c>
     </row>
     <row r="13">
-      <c r="I13" s="21"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="21"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14">
-      <c r="E14" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="I14" s="21"/>
-      <c r="K14" s="21"/>
+      <c r="E14" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="19"/>
+      <c r="K14" s="19"/>
     </row>
     <row r="15">
-      <c r="F15" s="23"/>
-      <c r="G15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="K15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="19"/>
+      <c r="I15" s="19"/>
+      <c r="K15" s="19"/>
     </row>
     <row r="16">
-      <c r="G16" s="22">
+      <c r="G16" s="20">
         <v>10</v>
       </c>
-      <c r="H16" s="24"/>
-      <c r="I16" s="21"/>
-      <c r="K16" s="21"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="19"/>
+      <c r="K16" s="19"/>
     </row>
     <row r="17">
-      <c r="C17" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="G17" s="21"/>
-      <c r="K17" s="21"/>
+      <c r="C17" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="19"/>
+      <c r="K17" s="19"/>
     </row>
     <row r="18">
-      <c r="D18" s="23"/>
-      <c r="E18" s="22">
+      <c r="D18" s="21"/>
+      <c r="E18" s="20">
         <v>2</v>
       </c>
-      <c r="F18" s="24"/>
-      <c r="G18" s="21"/>
-      <c r="K18" s="21"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="19"/>
+      <c r="K18" s="19"/>
     </row>
     <row r="19">
-      <c r="C19" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="21"/>
-      <c r="K19" s="21"/>
+      <c r="C19" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="22"/>
+      <c r="E19" s="19"/>
+      <c r="K19" s="19"/>
     </row>
     <row r="20">
-      <c r="K20" s="22">
+      <c r="K20" s="20">
         <v>21</v>
       </c>
     </row>
     <row r="21">
-      <c r="K21" s="21"/>
+      <c r="K21" s="19"/>
     </row>
     <row r="22">
-      <c r="E22" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="K22" s="21"/>
+      <c r="E22" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="K22" s="19"/>
     </row>
     <row r="23">
-      <c r="F23" s="23"/>
-      <c r="G23" s="21"/>
-      <c r="K23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="19"/>
+      <c r="K23" s="19"/>
     </row>
     <row r="24">
-      <c r="G24" s="22">
+      <c r="G24" s="20">
         <v>11</v>
       </c>
-      <c r="K24" s="21"/>
+      <c r="K24" s="19"/>
     </row>
     <row r="25">
-      <c r="C25" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="G25" s="21"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="21"/>
-      <c r="K25" s="21"/>
+      <c r="C25" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="G25" s="19"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="19"/>
+      <c r="K25" s="19"/>
     </row>
     <row r="26">
-      <c r="D26" s="23"/>
-      <c r="E26" s="22">
+      <c r="D26" s="21"/>
+      <c r="E26" s="20">
         <v>3</v>
       </c>
-      <c r="F26" s="24"/>
-      <c r="G26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="K26" s="21"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="K26" s="19"/>
     </row>
     <row r="27">
-      <c r="C27" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="21"/>
-      <c r="I27" s="21"/>
-      <c r="K27" s="21"/>
+      <c r="C27" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="22"/>
+      <c r="E27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="K27" s="19"/>
     </row>
     <row r="28">
-      <c r="I28" s="22">
+      <c r="I28" s="20">
         <v>18</v>
       </c>
-      <c r="J28" s="24"/>
-      <c r="K28" s="21"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="19"/>
     </row>
     <row r="29">
-      <c r="I29" s="21"/>
+      <c r="I29" s="19"/>
     </row>
     <row r="30">
-      <c r="E30" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="I30" s="21"/>
+      <c r="E30" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="I30" s="19"/>
     </row>
     <row r="31">
-      <c r="F31" s="23"/>
-      <c r="G31" s="21"/>
-      <c r="I31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="19"/>
+      <c r="I31" s="19"/>
     </row>
     <row r="32">
-      <c r="G32" s="22">
+      <c r="G32" s="20">
         <v>12</v>
       </c>
-      <c r="H32" s="24"/>
-      <c r="I32" s="21"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33">
-      <c r="C33" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G33" s="21"/>
+      <c r="C33" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="19"/>
     </row>
     <row r="34">
-      <c r="D34" s="23"/>
-      <c r="E34" s="22">
+      <c r="D34" s="21"/>
+      <c r="E34" s="20">
         <v>4</v>
       </c>
-      <c r="F34" s="24"/>
-      <c r="G34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="19"/>
     </row>
     <row r="35">
-      <c r="C35" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="D35" s="24"/>
-      <c r="E35" s="21"/>
+      <c r="C35" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" s="22"/>
+      <c r="E35" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2595,220 +2566,220 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="str">
+      <c r="A1" s="18" t="str">
         <f>IF(data!$B$1="","Shiaijo B",data!$B$1&amp;" - Shiaijo B")</f>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
     </row>
     <row r="6">
-      <c r="E6" s="25" t="s">
-        <v>53</v>
+      <c r="E6" s="23" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="7">
-      <c r="F7" s="23"/>
-      <c r="G7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="19"/>
     </row>
     <row r="8">
-      <c r="G8" s="22">
+      <c r="G8" s="20">
         <v>13</v>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="21"/>
+      <c r="C9" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="19"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10">
-      <c r="D10" s="23"/>
-      <c r="E10" s="22">
+      <c r="D10" s="21"/>
+      <c r="E10" s="20">
         <v>5</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="21"/>
-      <c r="I10" s="21"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11">
-      <c r="C11" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="21"/>
-      <c r="I11" s="21"/>
+      <c r="C11" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="22"/>
+      <c r="E11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12">
-      <c r="I12" s="22">
+      <c r="I12" s="20">
         <v>19</v>
       </c>
     </row>
     <row r="13">
-      <c r="I13" s="21"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="21"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14">
-      <c r="E14" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="I14" s="21"/>
-      <c r="K14" s="21"/>
+      <c r="E14" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="19"/>
+      <c r="K14" s="19"/>
     </row>
     <row r="15">
-      <c r="F15" s="23"/>
-      <c r="G15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="K15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="19"/>
+      <c r="I15" s="19"/>
+      <c r="K15" s="19"/>
     </row>
     <row r="16">
-      <c r="G16" s="22">
+      <c r="G16" s="20">
         <v>14</v>
       </c>
-      <c r="H16" s="24"/>
-      <c r="I16" s="21"/>
-      <c r="K16" s="21"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="19"/>
+      <c r="K16" s="19"/>
     </row>
     <row r="17">
-      <c r="C17" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="G17" s="21"/>
-      <c r="K17" s="21"/>
+      <c r="C17" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" s="19"/>
+      <c r="K17" s="19"/>
     </row>
     <row r="18">
-      <c r="D18" s="23"/>
-      <c r="E18" s="22">
+      <c r="D18" s="21"/>
+      <c r="E18" s="20">
         <v>6</v>
       </c>
-      <c r="F18" s="24"/>
-      <c r="G18" s="21"/>
-      <c r="K18" s="21"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="19"/>
+      <c r="K18" s="19"/>
     </row>
     <row r="19">
-      <c r="C19" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="21"/>
-      <c r="K19" s="21"/>
+      <c r="C19" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="22"/>
+      <c r="E19" s="19"/>
+      <c r="K19" s="19"/>
     </row>
     <row r="20">
-      <c r="K20" s="22">
+      <c r="K20" s="20">
         <v>22</v>
       </c>
     </row>
     <row r="21">
-      <c r="K21" s="21"/>
+      <c r="K21" s="19"/>
     </row>
     <row r="22">
-      <c r="E22" s="25" t="s">
+      <c r="E22" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22" s="19"/>
+    </row>
+    <row r="23">
+      <c r="F23" s="21"/>
+      <c r="G23" s="19"/>
+      <c r="K23" s="19"/>
+    </row>
+    <row r="24">
+      <c r="G24" s="20">
+        <v>15</v>
+      </c>
+      <c r="K24" s="19"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" s="19"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="19"/>
+      <c r="K25" s="19"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="21"/>
+      <c r="E26" s="20">
+        <v>7</v>
+      </c>
+      <c r="F26" s="22"/>
+      <c r="G26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="K26" s="19"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="22"/>
+      <c r="E27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="K27" s="19"/>
+    </row>
+    <row r="28">
+      <c r="I28" s="20">
         <v>20</v>
       </c>
-      <c r="K22" s="21"/>
-    </row>
-    <row r="23">
-      <c r="F23" s="23"/>
-      <c r="G23" s="21"/>
-      <c r="K23" s="21"/>
-    </row>
-    <row r="24">
-      <c r="G24" s="22">
-        <v>15</v>
-      </c>
-      <c r="K24" s="21"/>
-    </row>
-    <row r="25">
-      <c r="C25" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="G25" s="21"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="21"/>
-      <c r="K25" s="21"/>
-    </row>
-    <row r="26">
-      <c r="D26" s="23"/>
-      <c r="E26" s="22">
-        <v>7</v>
-      </c>
-      <c r="F26" s="24"/>
-      <c r="G26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="K26" s="21"/>
-    </row>
-    <row r="27">
-      <c r="C27" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="21"/>
-      <c r="I27" s="21"/>
-      <c r="K27" s="21"/>
-    </row>
-    <row r="28">
-      <c r="I28" s="22">
-        <v>20</v>
-      </c>
-      <c r="J28" s="24"/>
-      <c r="K28" s="21"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="19"/>
     </row>
     <row r="29">
-      <c r="I29" s="21"/>
+      <c r="I29" s="19"/>
     </row>
     <row r="30">
-      <c r="E30" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="I30" s="21"/>
+      <c r="E30" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="I30" s="19"/>
     </row>
     <row r="31">
-      <c r="F31" s="23"/>
-      <c r="G31" s="21"/>
-      <c r="I31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="19"/>
+      <c r="I31" s="19"/>
     </row>
     <row r="32">
-      <c r="G32" s="22">
+      <c r="G32" s="20">
         <v>16</v>
       </c>
-      <c r="H32" s="24"/>
-      <c r="I32" s="21"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="19"/>
     </row>
     <row r="33">
-      <c r="C33" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="G33" s="21"/>
+      <c r="C33" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="G33" s="19"/>
     </row>
     <row r="34">
-      <c r="D34" s="23"/>
-      <c r="E34" s="22">
+      <c r="D34" s="21"/>
+      <c r="E34" s="20">
         <v>8</v>
       </c>
-      <c r="F34" s="24"/>
-      <c r="G34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="19"/>
     </row>
     <row r="35">
-      <c r="C35" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" s="24"/>
-      <c r="E35" s="21"/>
+      <c r="C35" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="D35" s="22"/>
+      <c r="E35" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2832,28 +2803,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="51">
       <c r="A1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>8</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="11" customFormat="true" ht="16">
@@ -2879,8 +2850,8 @@
       <c r="G2" s="12">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="H2" s="12">
-        <f>E2+(A2*C2*F2)+G2</f>
+      <c r="H2" s="12" t="str">
+        <f>C2*I2+J2</f>
         <v>6.041666666666666E-2</v>
       </c>
     </row>
@@ -2944,26 +2915,26 @@
     </row>
     <row r="7" spans="1:8" ht="51">
       <c r="A7" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="G7" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="H7" s="13" t="s">
         <v>8</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="11" customFormat="true" ht="16">
@@ -3021,13 +2992,90 @@
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
     </row>
+    <row r="13">
+      <c r="E13" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>2</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26" t="str">
+        <f>H2</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26" t="str">
+        <f>H8</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26" t="str">
+        <f>H14+H15</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26" t="str">
+        <f>H16/A14</f>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="29">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="29" t="str">
+        <f>H18+H17</f>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E13:H13"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D4E4C4-15C1-724B-94C9-DD9C94F4D3CF}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
@@ -3046,1104 +3094,1036 @@
     <col max="16384" min="17" style="7" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="17" thickBot="true">
-      <c r="A1" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
+    <row r="1" spans="1:15">
+      <c r="A1" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="I2" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="I3" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
+      <c r="A3" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="I3" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L3" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O3" s="27" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G4" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I4" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O4" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="28" t="str">
+      <c r="A4" s="26" t="str">
         <f>'data'!$B$5</f>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28" t="str">
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26" t="str">
         <f>'data'!$B$4</f>
       </c>
-      <c r="I5" s="28" t="str">
-        <f>'data'!$B$8</f>
-      </c>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28" t="str">
-        <f>'data'!$B$7</f>
-      </c>
+      <c r="I4" s="26" t="str">
+        <f>'data'!$B$17</f>
+      </c>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26" t="str">
+        <f>'data'!$B$16</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="22"/>
+      <c r="N6" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="O6" s="22"/>
     </row>
     <row r="7">
       <c r="F7" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="22"/>
+      <c r="N7" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O7" s="22"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="I10" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G7" s="24"/>
-      <c r="N7" s="7" t="s">
+      <c r="I11" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L11" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O11" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O7" s="24"/>
-    </row>
-    <row r="8">
-      <c r="F8" s="7" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="str">
+        <f>'data'!$B$8</f>
+      </c>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26" t="str">
+        <f>'data'!$B$7</f>
+      </c>
+      <c r="I12" s="26" t="str">
+        <f>'data'!$B$20</f>
+      </c>
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="26"/>
+      <c r="M12" s="26"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="26" t="str">
+        <f>'data'!$B$19</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="F14" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="N8" s="7" t="s">
+      <c r="G14" s="22"/>
+      <c r="N14" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="O8" s="24"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="I11" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="20"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G12" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L12" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O12" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="28" t="str">
-        <f>'data'!$B$12</f>
-      </c>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28" t="str">
-        <f>'data'!$B$10</f>
-      </c>
-      <c r="I13" s="28" t="str">
-        <f>'data'!$B$14</f>
-      </c>
-      <c r="J13" s="28"/>
-      <c r="K13" s="28"/>
-      <c r="L13" s="28"/>
-      <c r="M13" s="28"/>
-      <c r="N13" s="28"/>
-      <c r="O13" s="28" t="str">
-        <f>'data'!$B$13</f>
-      </c>
+      <c r="O14" s="22"/>
     </row>
     <row r="15">
       <c r="F15" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" s="22"/>
+      <c r="N15" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O15" s="22"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="I18" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G15" s="24"/>
-      <c r="N15" s="7" t="s">
+      <c r="I19" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L19" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O19" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O15" s="24"/>
-    </row>
-    <row r="16">
-      <c r="F16" s="7" t="s">
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="str">
+        <f>'data'!$B$12</f>
+      </c>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26" t="str">
+        <f>'data'!$B$10</f>
+      </c>
+      <c r="I20" s="26" t="str">
+        <f>'data'!$B$23</f>
+      </c>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26" t="str">
+        <f>'data'!$B$22</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="F22" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G16" s="24"/>
-      <c r="N16" s="7" t="s">
+      <c r="G22" s="22"/>
+      <c r="N22" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="O16" s="24"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="20" t="s">
-        <v>95</v>
-      </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="I19" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="20"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G20" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I20" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L20" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O20" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="28" t="str">
-        <f>'data'!$B$17</f>
-      </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28" t="str">
-        <f>'data'!$B$16</f>
-      </c>
-      <c r="I21" s="28" t="str">
-        <f>'data'!$B$20</f>
-      </c>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28" t="str">
-        <f>'data'!$B$19</f>
-      </c>
+      <c r="O22" s="22"/>
     </row>
     <row r="23">
       <c r="F23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" s="22"/>
+      <c r="N23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O23" s="22"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="I26" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+      <c r="L26" s="18"/>
+      <c r="M26" s="18"/>
+      <c r="N26" s="18"/>
+      <c r="O26" s="18"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G27" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G23" s="24"/>
-      <c r="N23" s="7" t="s">
+      <c r="I27" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L27" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O27" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O23" s="24"/>
-    </row>
-    <row r="24">
-      <c r="F24" s="7" t="s">
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="str">
+        <f>'data'!$B$14</f>
+      </c>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26" t="str">
+        <f>'data'!$B$13</f>
+      </c>
+      <c r="I28" s="26" t="str">
+        <f>'data'!$B$26</f>
+      </c>
+      <c r="J28" s="26"/>
+      <c r="K28" s="26"/>
+      <c r="L28" s="26"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+      <c r="O28" s="26" t="str">
+        <f>'data'!$B$25</f>
+      </c>
+    </row>
+    <row r="30">
+      <c r="F30" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G24" s="24"/>
-      <c r="N24" s="7" t="s">
+      <c r="G30" s="22"/>
+      <c r="N30" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="O24" s="24"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="I27" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
-      <c r="L27" s="20"/>
-      <c r="M27" s="20"/>
-      <c r="N27" s="20"/>
-      <c r="O27" s="20"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D28" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G28" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I28" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L28" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O28" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="28" t="str">
-        <f>'data'!$B$23</f>
-      </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28" t="str">
-        <f>'data'!$B$22</f>
-      </c>
-      <c r="I29" s="28" t="str">
-        <f>'data'!$B$26</f>
-      </c>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28" t="str">
-        <f>'data'!$B$25</f>
-      </c>
+      <c r="O30" s="22"/>
     </row>
     <row r="31">
       <c r="F31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="22"/>
+      <c r="N31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O31" s="22"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="I39" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="18"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="18"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D40" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G40" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G31" s="24"/>
-      <c r="N31" s="7" t="s">
+      <c r="I40" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L40" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O40" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O31" s="24"/>
-    </row>
-    <row r="32">
-      <c r="F32" s="7" t="s">
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="str">
+        <f>CONCATENATE("M 1 ",'Elimination Matches'!G6)</f>
+      </c>
+      <c r="B41" s="26"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="26" t="str">
+        <f>'data'!$B$21</f>
+      </c>
+      <c r="I41" s="26" t="str">
+        <f>CONCATENATE("M 5 ",'Elimination Matches'!O6)</f>
+      </c>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
+      <c r="N41" s="26"/>
+      <c r="O41" s="26" t="str">
+        <f>'data'!$B$15</f>
+      </c>
+    </row>
+    <row r="43">
+      <c r="F43" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G32" s="24"/>
-      <c r="N32" s="7" t="s">
+      <c r="G43" s="22"/>
+      <c r="N43" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="O32" s="24"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="20"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="I42" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
-      <c r="L42" s="20"/>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-      <c r="O42" s="20"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D43" s="28" t="s">
+      <c r="O43" s="22"/>
+    </row>
+    <row r="44">
+      <c r="F44" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G44" s="22"/>
+      <c r="N44" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O44" s="22"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+      <c r="I47" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="J47" s="18"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="18"/>
+      <c r="M47" s="18"/>
+      <c r="N47" s="18"/>
+      <c r="O47" s="18"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="G43" s="29" t="s">
+      <c r="D48" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="I43" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L43" s="28" t="s">
+      <c r="G48" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="I48" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="O43" s="29" t="s">
+      <c r="L48" s="26" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="28" t="str">
-        <f>CONCATENATE("M 1 ",'Elimination Matches'!G7)</f>
-      </c>
-      <c r="B44" s="28"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="28"/>
-      <c r="G44" s="28" t="str">
+      <c r="O48" s="27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="str">
+        <f>CONCATENATE("M 2 ",'Elimination Matches'!G14)</f>
+      </c>
+      <c r="B49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26" t="str">
+        <f>'data'!$B$6</f>
+      </c>
+      <c r="I49" s="26" t="str">
+        <f>CONCATENATE("M 6 ",'Elimination Matches'!O14)</f>
+      </c>
+      <c r="J49" s="26"/>
+      <c r="K49" s="26"/>
+      <c r="L49" s="26"/>
+      <c r="M49" s="26"/>
+      <c r="N49" s="26"/>
+      <c r="O49" s="26" t="str">
+        <f>'data'!$B$18</f>
+      </c>
+    </row>
+    <row r="51">
+      <c r="F51" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G51" s="22"/>
+      <c r="N51" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="O51" s="22"/>
+    </row>
+    <row r="52">
+      <c r="F52" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="22"/>
+      <c r="N52" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O52" s="22"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+      <c r="I55" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="J55" s="18"/>
+      <c r="K55" s="18"/>
+      <c r="L55" s="18"/>
+      <c r="M55" s="18"/>
+      <c r="N55" s="18"/>
+      <c r="O55" s="18"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D56" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G56" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="I56" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L56" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O56" s="27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="26" t="str">
+        <f>CONCATENATE("M 3 ",'Elimination Matches'!G22)</f>
+      </c>
+      <c r="B57" s="26"/>
+      <c r="C57" s="26"/>
+      <c r="D57" s="26"/>
+      <c r="E57" s="26"/>
+      <c r="F57" s="26"/>
+      <c r="G57" s="26" t="str">
+        <f>'data'!$B$9</f>
+      </c>
+      <c r="I57" s="26" t="str">
+        <f>CONCATENATE("M 7 ",'Elimination Matches'!O22)</f>
+      </c>
+      <c r="J57" s="26"/>
+      <c r="K57" s="26"/>
+      <c r="L57" s="26"/>
+      <c r="M57" s="26"/>
+      <c r="N57" s="26"/>
+      <c r="O57" s="26" t="str">
         <f>'data'!$B$21</f>
       </c>
-      <c r="I44" s="28" t="str">
-        <f>CONCATENATE("M 2 ",'Elimination Matches'!O7)</f>
-      </c>
-      <c r="J44" s="28"/>
-      <c r="K44" s="28"/>
-      <c r="L44" s="28"/>
-      <c r="M44" s="28"/>
-      <c r="N44" s="28"/>
-      <c r="O44" s="28" t="str">
-        <f>'data'!$B$6</f>
-      </c>
-    </row>
-    <row r="46">
-      <c r="F46" s="7" t="s">
+    </row>
+    <row r="59">
+      <c r="F59" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G59" s="22"/>
+      <c r="N59" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="O59" s="22"/>
+    </row>
+    <row r="60">
+      <c r="F60" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G60" s="22"/>
+      <c r="N60" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O60" s="22"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+      <c r="F63" s="18"/>
+      <c r="G63" s="18"/>
+      <c r="I63" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="J63" s="18"/>
+      <c r="K63" s="18"/>
+      <c r="L63" s="18"/>
+      <c r="M63" s="18"/>
+      <c r="N63" s="18"/>
+      <c r="O63" s="18"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D64" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G64" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G46" s="24"/>
-      <c r="N46" s="7" t="s">
+      <c r="I64" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L64" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O64" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O46" s="24"/>
-    </row>
-    <row r="47">
-      <c r="F47" s="7" t="s">
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="str">
+        <f>CONCATENATE("M 4 ",'Elimination Matches'!G30)</f>
+      </c>
+      <c r="B65" s="26"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="26"/>
+      <c r="F65" s="26"/>
+      <c r="G65" s="26" t="str">
+        <f>'data'!$B$12</f>
+      </c>
+      <c r="I65" s="26" t="str">
+        <f>CONCATENATE("M 8 ",'Elimination Matches'!O30)</f>
+      </c>
+      <c r="J65" s="26"/>
+      <c r="K65" s="26"/>
+      <c r="L65" s="26"/>
+      <c r="M65" s="26"/>
+      <c r="N65" s="26"/>
+      <c r="O65" s="26" t="str">
+        <f>'data'!$B$24</f>
+      </c>
+    </row>
+    <row r="67">
+      <c r="F67" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G47" s="24"/>
-      <c r="N47" s="7" t="s">
+      <c r="G67" s="22"/>
+      <c r="N67" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="O47" s="24"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="20"/>
-      <c r="F50" s="20"/>
-      <c r="G50" s="20"/>
-      <c r="I50" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20"/>
-      <c r="L50" s="20"/>
-      <c r="M50" s="20"/>
-      <c r="N50" s="20"/>
-      <c r="O50" s="20"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D51" s="28" t="s">
+      <c r="O67" s="22"/>
+    </row>
+    <row r="68">
+      <c r="F68" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G68" s="22"/>
+      <c r="N68" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O68" s="22"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B76" s="18"/>
+      <c r="C76" s="18"/>
+      <c r="D76" s="18"/>
+      <c r="E76" s="18"/>
+      <c r="F76" s="18"/>
+      <c r="G76" s="18"/>
+      <c r="I76" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="J76" s="18"/>
+      <c r="K76" s="18"/>
+      <c r="L76" s="18"/>
+      <c r="M76" s="18"/>
+      <c r="N76" s="18"/>
+      <c r="O76" s="18"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="G51" s="29" t="s">
+      <c r="D77" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="I51" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L51" s="28" t="s">
+      <c r="G77" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="I77" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="O51" s="29" t="s">
+      <c r="L77" s="26" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="28" t="str">
-        <f>CONCATENATE("M 3 ",'Elimination Matches'!G15)</f>
-      </c>
-      <c r="B52" s="28"/>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="28"/>
-      <c r="G52" s="28" t="str">
-        <f>'data'!$B$9</f>
-      </c>
-      <c r="I52" s="28" t="str">
-        <f>CONCATENATE("M 4 ",'Elimination Matches'!O15)</f>
-      </c>
-      <c r="J52" s="28"/>
-      <c r="K52" s="28"/>
-      <c r="L52" s="28"/>
-      <c r="M52" s="28"/>
-      <c r="N52" s="28"/>
-      <c r="O52" s="28" t="str">
-        <f>'data'!$B$12</f>
-      </c>
-    </row>
-    <row r="54">
-      <c r="F54" s="7" t="s">
+      <c r="O77" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G54" s="24"/>
-      <c r="N54" s="7" t="s">
+    </row>
+    <row r="78">
+      <c r="A78" s="26" t="str">
+        <f>CONCATENATE("M 10 ",'Elimination Matches'!G51)</f>
+      </c>
+      <c r="B78" s="26"/>
+      <c r="C78" s="26"/>
+      <c r="D78" s="26"/>
+      <c r="E78" s="26"/>
+      <c r="F78" s="26"/>
+      <c r="G78" s="26" t="str">
+        <f>CONCATENATE("M 9 ",'Elimination Matches'!G43)</f>
+      </c>
+      <c r="I78" s="26" t="str">
+        <f>CONCATENATE("M 14 ",'Elimination Matches'!O51)</f>
+      </c>
+      <c r="J78" s="26"/>
+      <c r="K78" s="26"/>
+      <c r="L78" s="26"/>
+      <c r="M78" s="26"/>
+      <c r="N78" s="26"/>
+      <c r="O78" s="26" t="str">
+        <f>CONCATENATE("M 13 ",'Elimination Matches'!O43)</f>
+      </c>
+    </row>
+    <row r="80">
+      <c r="F80" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G80" s="22"/>
+      <c r="N80" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="O80" s="22"/>
+    </row>
+    <row r="81">
+      <c r="F81" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G81" s="22"/>
+      <c r="N81" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O81" s="22"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B84" s="18"/>
+      <c r="C84" s="18"/>
+      <c r="D84" s="18"/>
+      <c r="E84" s="18"/>
+      <c r="F84" s="18"/>
+      <c r="G84" s="18"/>
+      <c r="I84" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="J84" s="18"/>
+      <c r="K84" s="18"/>
+      <c r="L84" s="18"/>
+      <c r="M84" s="18"/>
+      <c r="N84" s="18"/>
+      <c r="O84" s="18"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D85" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G85" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O54" s="24"/>
-    </row>
-    <row r="55">
-      <c r="F55" s="7" t="s">
+      <c r="I85" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="L85" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="O85" s="27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="26" t="str">
+        <f>CONCATENATE("M 12 ",'Elimination Matches'!G67)</f>
+      </c>
+      <c r="B86" s="26"/>
+      <c r="C86" s="26"/>
+      <c r="D86" s="26"/>
+      <c r="E86" s="26"/>
+      <c r="F86" s="26"/>
+      <c r="G86" s="26" t="str">
+        <f>CONCATENATE("M 11 ",'Elimination Matches'!G59)</f>
+      </c>
+      <c r="I86" s="26" t="str">
+        <f>CONCATENATE("M 16 ",'Elimination Matches'!O67)</f>
+      </c>
+      <c r="J86" s="26"/>
+      <c r="K86" s="26"/>
+      <c r="L86" s="26"/>
+      <c r="M86" s="26"/>
+      <c r="N86" s="26"/>
+      <c r="O86" s="26" t="str">
+        <f>CONCATENATE("M 15 ",'Elimination Matches'!O59)</f>
+      </c>
+    </row>
+    <row r="88">
+      <c r="F88" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G55" s="24"/>
-      <c r="N55" s="7" t="s">
+      <c r="G88" s="22"/>
+      <c r="N88" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="O55" s="24"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="B58" s="20"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="20"/>
-      <c r="I58" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="J58" s="20"/>
-      <c r="K58" s="20"/>
-      <c r="L58" s="20"/>
-      <c r="M58" s="20"/>
-      <c r="N58" s="20"/>
-      <c r="O58" s="20"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D59" s="28" t="s">
+      <c r="O88" s="22"/>
+    </row>
+    <row r="89">
+      <c r="F89" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G89" s="22"/>
+      <c r="N89" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O89" s="22"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B97" s="18"/>
+      <c r="C97" s="18"/>
+      <c r="D97" s="18"/>
+      <c r="E97" s="18"/>
+      <c r="F97" s="18"/>
+      <c r="G97" s="18"/>
+      <c r="I97" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="J97" s="18"/>
+      <c r="K97" s="18"/>
+      <c r="L97" s="18"/>
+      <c r="M97" s="18"/>
+      <c r="N97" s="18"/>
+      <c r="O97" s="18"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="G59" s="29" t="s">
+      <c r="D98" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="I59" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L59" s="28" t="s">
+      <c r="G98" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="I98" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="O59" s="29" t="s">
+      <c r="L98" s="26" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="28" t="str">
-        <f>CONCATENATE("M 5 ",'Elimination Matches'!G23)</f>
-      </c>
-      <c r="B60" s="28"/>
-      <c r="C60" s="28"/>
-      <c r="D60" s="28"/>
-      <c r="E60" s="28"/>
-      <c r="F60" s="28"/>
-      <c r="G60" s="28" t="str">
-        <f>'data'!$B$15</f>
-      </c>
-      <c r="I60" s="28" t="str">
-        <f>CONCATENATE("M 6 ",'Elimination Matches'!O23)</f>
-      </c>
-      <c r="J60" s="28"/>
-      <c r="K60" s="28"/>
-      <c r="L60" s="28"/>
-      <c r="M60" s="28"/>
-      <c r="N60" s="28"/>
-      <c r="O60" s="28" t="str">
-        <f>'data'!$B$18</f>
-      </c>
-    </row>
-    <row r="62">
-      <c r="F62" s="7" t="s">
+      <c r="O98" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="G62" s="24"/>
-      <c r="N62" s="7" t="s">
+    </row>
+    <row r="99">
+      <c r="A99" s="26" t="str">
+        <f>CONCATENATE("M 18 ",'Elimination Matches'!G88)</f>
+      </c>
+      <c r="B99" s="26"/>
+      <c r="C99" s="26"/>
+      <c r="D99" s="26"/>
+      <c r="E99" s="26"/>
+      <c r="F99" s="26"/>
+      <c r="G99" s="26" t="str">
+        <f>CONCATENATE("M 17 ",'Elimination Matches'!G80)</f>
+      </c>
+      <c r="I99" s="26" t="str">
+        <f>CONCATENATE("M 20 ",'Elimination Matches'!O88)</f>
+      </c>
+      <c r="J99" s="26"/>
+      <c r="K99" s="26"/>
+      <c r="L99" s="26"/>
+      <c r="M99" s="26"/>
+      <c r="N99" s="26"/>
+      <c r="O99" s="26" t="str">
+        <f>CONCATENATE("M 19 ",'Elimination Matches'!O80)</f>
+      </c>
+    </row>
+    <row r="101">
+      <c r="F101" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G101" s="22"/>
+      <c r="N101" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="O101" s="22"/>
+    </row>
+    <row r="102">
+      <c r="F102" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G102" s="22"/>
+      <c r="N102" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="O102" s="22"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="B110" s="18"/>
+      <c r="C110" s="18"/>
+      <c r="D110" s="18"/>
+      <c r="E110" s="18"/>
+      <c r="F110" s="18"/>
+      <c r="G110" s="18"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D111" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="G111" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="O62" s="24"/>
-    </row>
-    <row r="63">
-      <c r="F63" s="7" t="s">
+    </row>
+    <row r="112">
+      <c r="A112" s="26" t="str">
+        <f>CONCATENATE("M 22 ",'Elimination Matches'!O101)</f>
+      </c>
+      <c r="B112" s="26"/>
+      <c r="C112" s="26"/>
+      <c r="D112" s="26"/>
+      <c r="E112" s="26"/>
+      <c r="F112" s="26"/>
+      <c r="G112" s="26" t="str">
+        <f>CONCATENATE("M 21 ",'Elimination Matches'!G101)</f>
+      </c>
+    </row>
+    <row r="114">
+      <c r="F114" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G63" s="24"/>
-      <c r="N63" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="O63" s="24"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
-      <c r="E66" s="20"/>
-      <c r="F66" s="20"/>
-      <c r="G66" s="20"/>
-      <c r="I66" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="J66" s="20"/>
-      <c r="K66" s="20"/>
-      <c r="L66" s="20"/>
-      <c r="M66" s="20"/>
-      <c r="N66" s="20"/>
-      <c r="O66" s="20"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D67" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G67" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I67" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L67" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O67" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="28" t="str">
-        <f>CONCATENATE("M 7 ",'Elimination Matches'!G31)</f>
-      </c>
-      <c r="B68" s="28"/>
-      <c r="C68" s="28"/>
-      <c r="D68" s="28"/>
-      <c r="E68" s="28"/>
-      <c r="F68" s="28"/>
-      <c r="G68" s="28" t="str">
-        <f>'data'!$B$21</f>
-      </c>
-      <c r="I68" s="28" t="str">
-        <f>CONCATENATE("M 8 ",'Elimination Matches'!O31)</f>
-      </c>
-      <c r="J68" s="28"/>
-      <c r="K68" s="28"/>
-      <c r="L68" s="28"/>
-      <c r="M68" s="28"/>
-      <c r="N68" s="28"/>
-      <c r="O68" s="28" t="str">
-        <f>'data'!$B$24</f>
-      </c>
-    </row>
-    <row r="70">
-      <c r="F70" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="G70" s="24"/>
-      <c r="N70" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="O70" s="24"/>
-    </row>
-    <row r="71">
-      <c r="F71" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G71" s="24"/>
-      <c r="N71" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="O71" s="24"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="B79" s="20"/>
-      <c r="C79" s="20"/>
-      <c r="D79" s="20"/>
-      <c r="E79" s="20"/>
-      <c r="F79" s="20"/>
-      <c r="G79" s="20"/>
-      <c r="H79" s="20"/>
-      <c r="I79" s="20"/>
-      <c r="J79" s="20"/>
-      <c r="K79" s="20"/>
-      <c r="L79" s="20"/>
-      <c r="M79" s="20"/>
-      <c r="N79" s="20"/>
-      <c r="O79" s="20"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="B81" s="20"/>
-      <c r="C81" s="20"/>
-      <c r="D81" s="20"/>
-      <c r="E81" s="20"/>
-      <c r="F81" s="20"/>
-      <c r="G81" s="20"/>
-      <c r="I81" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="J81" s="20"/>
-      <c r="K81" s="20"/>
-      <c r="L81" s="20"/>
-      <c r="M81" s="20"/>
-      <c r="N81" s="20"/>
-      <c r="O81" s="20"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D82" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G82" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I82" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L82" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O82" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="28" t="str">
-        <f>CONCATENATE("M 10 ",'Elimination Matches'!O46)</f>
-      </c>
-      <c r="B83" s="28"/>
-      <c r="C83" s="28"/>
-      <c r="D83" s="28"/>
-      <c r="E83" s="28"/>
-      <c r="F83" s="28"/>
-      <c r="G83" s="28" t="str">
-        <f>CONCATENATE("M 9 ",'Elimination Matches'!G46)</f>
-      </c>
-      <c r="I83" s="28" t="str">
-        <f>CONCATENATE("M 12 ",'Elimination Matches'!O54)</f>
-      </c>
-      <c r="J83" s="28"/>
-      <c r="K83" s="28"/>
-      <c r="L83" s="28"/>
-      <c r="M83" s="28"/>
-      <c r="N83" s="28"/>
-      <c r="O83" s="28" t="str">
-        <f>CONCATENATE("M 11 ",'Elimination Matches'!G54)</f>
-      </c>
-    </row>
-    <row r="85">
-      <c r="F85" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="G85" s="24"/>
-      <c r="N85" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="O85" s="24"/>
-    </row>
-    <row r="86">
-      <c r="F86" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G86" s="24"/>
-      <c r="N86" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="O86" s="24"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="B89" s="20"/>
-      <c r="C89" s="20"/>
-      <c r="D89" s="20"/>
-      <c r="E89" s="20"/>
-      <c r="F89" s="20"/>
-      <c r="G89" s="20"/>
-      <c r="I89" s="20" t="s">
-        <v>112</v>
-      </c>
-      <c r="J89" s="20"/>
-      <c r="K89" s="20"/>
-      <c r="L89" s="20"/>
-      <c r="M89" s="20"/>
-      <c r="N89" s="20"/>
-      <c r="O89" s="20"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D90" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G90" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I90" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L90" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O90" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="28" t="str">
-        <f>CONCATENATE("M 14 ",'Elimination Matches'!O62)</f>
-      </c>
-      <c r="B91" s="28"/>
-      <c r="C91" s="28"/>
-      <c r="D91" s="28"/>
-      <c r="E91" s="28"/>
-      <c r="F91" s="28"/>
-      <c r="G91" s="28" t="str">
-        <f>CONCATENATE("M 13 ",'Elimination Matches'!G62)</f>
-      </c>
-      <c r="I91" s="28" t="str">
-        <f>CONCATENATE("M 16 ",'Elimination Matches'!O70)</f>
-      </c>
-      <c r="J91" s="28"/>
-      <c r="K91" s="28"/>
-      <c r="L91" s="28"/>
-      <c r="M91" s="28"/>
-      <c r="N91" s="28"/>
-      <c r="O91" s="28" t="str">
-        <f>CONCATENATE("M 15 ",'Elimination Matches'!G70)</f>
-      </c>
-    </row>
-    <row r="93">
-      <c r="F93" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="G93" s="24"/>
-      <c r="N93" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="O93" s="24"/>
-    </row>
-    <row r="94">
-      <c r="F94" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G94" s="24"/>
-      <c r="N94" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="O94" s="24"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="B102" s="20"/>
-      <c r="C102" s="20"/>
-      <c r="D102" s="20"/>
-      <c r="E102" s="20"/>
-      <c r="F102" s="20"/>
-      <c r="G102" s="20"/>
-      <c r="H102" s="20"/>
-      <c r="I102" s="20"/>
-      <c r="J102" s="20"/>
-      <c r="K102" s="20"/>
-      <c r="L102" s="20"/>
-      <c r="M102" s="20"/>
-      <c r="N102" s="20"/>
-      <c r="O102" s="20"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="B104" s="20"/>
-      <c r="C104" s="20"/>
-      <c r="D104" s="20"/>
-      <c r="E104" s="20"/>
-      <c r="F104" s="20"/>
-      <c r="G104" s="20"/>
-      <c r="I104" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="J104" s="20"/>
-      <c r="K104" s="20"/>
-      <c r="L104" s="20"/>
-      <c r="M104" s="20"/>
-      <c r="N104" s="20"/>
-      <c r="O104" s="20"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D105" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G105" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I105" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="L105" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="O105" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="28" t="str">
-        <f>CONCATENATE("M 18 ",'Elimination Matches'!O85)</f>
-      </c>
-      <c r="B106" s="28"/>
-      <c r="C106" s="28"/>
-      <c r="D106" s="28"/>
-      <c r="E106" s="28"/>
-      <c r="F106" s="28"/>
-      <c r="G106" s="28" t="str">
-        <f>CONCATENATE("M 17 ",'Elimination Matches'!G85)</f>
-      </c>
-      <c r="I106" s="28" t="str">
-        <f>CONCATENATE("M 20 ",'Elimination Matches'!O93)</f>
-      </c>
-      <c r="J106" s="28"/>
-      <c r="K106" s="28"/>
-      <c r="L106" s="28"/>
-      <c r="M106" s="28"/>
-      <c r="N106" s="28"/>
-      <c r="O106" s="28" t="str">
-        <f>CONCATENATE("M 19 ",'Elimination Matches'!G93)</f>
-      </c>
-    </row>
-    <row r="108">
-      <c r="F108" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="G108" s="24"/>
-      <c r="N108" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="O108" s="24"/>
-    </row>
-    <row r="109">
-      <c r="F109" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G109" s="24"/>
-      <c r="N109" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="O109" s="24"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="B117" s="20"/>
-      <c r="C117" s="20"/>
-      <c r="D117" s="20"/>
-      <c r="E117" s="20"/>
-      <c r="F117" s="20"/>
-      <c r="G117" s="20"/>
-      <c r="H117" s="20"/>
-      <c r="I117" s="20"/>
-      <c r="J117" s="20"/>
-      <c r="K117" s="20"/>
-      <c r="L117" s="20"/>
-      <c r="M117" s="20"/>
-      <c r="N117" s="20"/>
-      <c r="O117" s="20"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="B119" s="20"/>
-      <c r="C119" s="20"/>
-      <c r="D119" s="20"/>
-      <c r="E119" s="20"/>
-      <c r="F119" s="20"/>
-      <c r="G119" s="20"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="D120" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="G120" s="29" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="28" t="str">
-        <f>CONCATENATE("M 22 ",'Elimination Matches'!O108)</f>
-      </c>
-      <c r="B121" s="28"/>
-      <c r="C121" s="28"/>
-      <c r="D121" s="28"/>
-      <c r="E121" s="28"/>
-      <c r="F121" s="28"/>
-      <c r="G121" s="28" t="str">
-        <f>CONCATENATE("M 21 ",'Elimination Matches'!G108)</f>
-      </c>
-    </row>
-    <row r="123">
-      <c r="F123" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="G123" s="24"/>
-    </row>
-    <row r="124">
-      <c r="F124" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G124" s="24"/>
+      <c r="G114" s="22"/>
+    </row>
+    <row r="115">
+      <c r="F115" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G115" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="I3:O3"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="I11:O11"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="I19:O19"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="I27:O27"/>
-    <mergeCell ref="A40:O40"/>
-    <mergeCell ref="A42:G42"/>
-    <mergeCell ref="I42:O42"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="I50:O50"/>
-    <mergeCell ref="A58:G58"/>
-    <mergeCell ref="I58:O58"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="I66:O66"/>
-    <mergeCell ref="A79:O79"/>
-    <mergeCell ref="A81:G81"/>
-    <mergeCell ref="I81:O81"/>
-    <mergeCell ref="A89:G89"/>
-    <mergeCell ref="I89:O89"/>
-    <mergeCell ref="A102:O102"/>
-    <mergeCell ref="A104:G104"/>
-    <mergeCell ref="I104:O104"/>
-    <mergeCell ref="A117:O117"/>
-    <mergeCell ref="A119:G119"/>
+  <mergeCells count="25">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="I2:O2"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="I10:O10"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="I18:O18"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="I26:O26"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="I39:O39"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="I47:O47"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="I55:O55"/>
+    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="I63:O63"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="I76:O76"/>
+    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="I84:O84"/>
+    <mergeCell ref="A97:G97"/>
+    <mergeCell ref="I97:O97"/>
+    <mergeCell ref="A110:G110"/>
   </mergeCells>
+  <printOptions horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" fitToWidth="2" orientation="portrait" pageOrder="downThenOver" paperSize="9"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="38" max="16383" man="true"/>
+    <brk id="75" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks count="1" manualBreakCount="1">
+    <brk id="8" max="1048575" man="true"/>
+  </colBreaks>
 </worksheet>
 </file>
 
@@ -4161,292 +4141,292 @@
   </cols>
   <sheetData>
     <row r="1" ht="110" customHeight="true">
-      <c r="A1" s="26">
+      <c r="A1" s="24">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="str">
+      <c r="B1" s="25" t="str">
         <f>data!D3</f>
       </c>
     </row>
     <row r="2" ht="115" customHeight="true">
-      <c r="A2" s="26"/>
-      <c r="B2" s="27"/>
+      <c r="A2" s="24"/>
+      <c r="B2" s="25"/>
     </row>
     <row r="3" ht="110" customHeight="true">
-      <c r="A3" s="26">
+      <c r="A3" s="24">
         <v>1</v>
       </c>
-      <c r="B3" s="27" t="str">
+      <c r="B3" s="25" t="str">
         <f>data!D4</f>
       </c>
     </row>
     <row r="4" ht="115" customHeight="true">
-      <c r="A4" s="26"/>
-      <c r="B4" s="27"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="25"/>
     </row>
     <row r="5" ht="110" customHeight="true">
-      <c r="A5" s="26">
+      <c r="A5" s="24">
         <v>2</v>
       </c>
-      <c r="B5" s="27" t="str">
+      <c r="B5" s="25" t="str">
         <f>data!D5</f>
       </c>
     </row>
     <row r="6" ht="115" customHeight="true">
-      <c r="A6" s="26"/>
-      <c r="B6" s="27"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="25"/>
     </row>
     <row r="7" ht="110" customHeight="true">
-      <c r="A7" s="26">
+      <c r="A7" s="24">
         <v>3</v>
       </c>
-      <c r="B7" s="27" t="str">
+      <c r="B7" s="25" t="str">
         <f>data!D6</f>
       </c>
     </row>
     <row r="8" ht="115" customHeight="true">
-      <c r="A8" s="26"/>
-      <c r="B8" s="27"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="25"/>
     </row>
     <row r="9" ht="110" customHeight="true">
-      <c r="A9" s="26">
+      <c r="A9" s="24">
         <v>4</v>
       </c>
-      <c r="B9" s="27" t="str">
+      <c r="B9" s="25" t="str">
         <f>data!D7</f>
       </c>
     </row>
     <row r="10" ht="115" customHeight="true">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
     </row>
     <row r="11" ht="110" customHeight="true">
-      <c r="A11" s="26">
+      <c r="A11" s="24">
         <v>5</v>
       </c>
-      <c r="B11" s="27" t="str">
+      <c r="B11" s="25" t="str">
         <f>data!D8</f>
       </c>
     </row>
     <row r="12" ht="115" customHeight="true">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="25"/>
     </row>
     <row r="13" ht="110" customHeight="true">
-      <c r="A13" s="26">
+      <c r="A13" s="24">
         <v>6</v>
       </c>
-      <c r="B13" s="27" t="str">
+      <c r="B13" s="25" t="str">
         <f>data!D9</f>
       </c>
     </row>
     <row r="14" ht="115" customHeight="true">
-      <c r="A14" s="26"/>
-      <c r="B14" s="27"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="25"/>
     </row>
     <row r="15" ht="110" customHeight="true">
-      <c r="A15" s="26">
+      <c r="A15" s="24">
         <v>7</v>
       </c>
-      <c r="B15" s="27" t="str">
+      <c r="B15" s="25" t="str">
         <f>data!D10</f>
       </c>
     </row>
     <row r="16" ht="115" customHeight="true">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="25"/>
     </row>
     <row r="17" ht="110" customHeight="true">
-      <c r="A17" s="26">
+      <c r="A17" s="24">
         <v>8</v>
       </c>
-      <c r="B17" s="27" t="str">
+      <c r="B17" s="25" t="str">
         <f>data!D11</f>
       </c>
     </row>
     <row r="18" ht="115" customHeight="true">
-      <c r="A18" s="26"/>
-      <c r="B18" s="27"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="25"/>
     </row>
     <row r="19" ht="110" customHeight="true">
-      <c r="A19" s="26">
+      <c r="A19" s="24">
         <v>9</v>
       </c>
-      <c r="B19" s="27" t="str">
+      <c r="B19" s="25" t="str">
         <f>data!D12</f>
       </c>
     </row>
     <row r="20" ht="115" customHeight="true">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="25"/>
     </row>
     <row r="21" ht="110" customHeight="true">
-      <c r="A21" s="26">
+      <c r="A21" s="24">
         <v>10</v>
       </c>
-      <c r="B21" s="27" t="str">
+      <c r="B21" s="25" t="str">
         <f>data!D13</f>
       </c>
     </row>
     <row r="22" ht="115" customHeight="true">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="25"/>
     </row>
     <row r="23" ht="110" customHeight="true">
-      <c r="A23" s="26">
+      <c r="A23" s="24">
         <v>11</v>
       </c>
-      <c r="B23" s="27" t="str">
+      <c r="B23" s="25" t="str">
         <f>data!D14</f>
       </c>
     </row>
     <row r="24" ht="115" customHeight="true">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="25"/>
     </row>
     <row r="25" ht="110" customHeight="true">
-      <c r="A25" s="26">
+      <c r="A25" s="24">
         <v>12</v>
       </c>
-      <c r="B25" s="27" t="str">
+      <c r="B25" s="25" t="str">
         <f>data!D15</f>
       </c>
     </row>
     <row r="26" ht="115" customHeight="true">
-      <c r="A26" s="26"/>
-      <c r="B26" s="27"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="25"/>
     </row>
     <row r="27" ht="110" customHeight="true">
-      <c r="A27" s="26">
+      <c r="A27" s="24">
         <v>13</v>
       </c>
-      <c r="B27" s="27" t="str">
+      <c r="B27" s="25" t="str">
         <f>data!D16</f>
       </c>
     </row>
     <row r="28" ht="115" customHeight="true">
-      <c r="A28" s="26"/>
-      <c r="B28" s="27"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="25"/>
     </row>
     <row r="29" ht="110" customHeight="true">
-      <c r="A29" s="26">
+      <c r="A29" s="24">
         <v>14</v>
       </c>
-      <c r="B29" s="27" t="str">
+      <c r="B29" s="25" t="str">
         <f>data!D17</f>
       </c>
     </row>
     <row r="30" ht="115" customHeight="true">
-      <c r="A30" s="26"/>
-      <c r="B30" s="27"/>
+      <c r="A30" s="24"/>
+      <c r="B30" s="25"/>
     </row>
     <row r="31" ht="110" customHeight="true">
-      <c r="A31" s="26">
+      <c r="A31" s="24">
         <v>15</v>
       </c>
-      <c r="B31" s="27" t="str">
+      <c r="B31" s="25" t="str">
         <f>data!D18</f>
       </c>
     </row>
     <row r="32" ht="115" customHeight="true">
-      <c r="A32" s="26"/>
-      <c r="B32" s="27"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="25"/>
     </row>
     <row r="33" ht="110" customHeight="true">
-      <c r="A33" s="26">
+      <c r="A33" s="24">
         <v>16</v>
       </c>
-      <c r="B33" s="27" t="str">
+      <c r="B33" s="25" t="str">
         <f>data!D19</f>
       </c>
     </row>
     <row r="34" ht="115" customHeight="true">
-      <c r="A34" s="26"/>
-      <c r="B34" s="27"/>
+      <c r="A34" s="24"/>
+      <c r="B34" s="25"/>
     </row>
     <row r="35" ht="110" customHeight="true">
-      <c r="A35" s="26">
+      <c r="A35" s="24">
         <v>17</v>
       </c>
-      <c r="B35" s="27" t="str">
+      <c r="B35" s="25" t="str">
         <f>data!D20</f>
       </c>
     </row>
     <row r="36" ht="115" customHeight="true">
-      <c r="A36" s="26"/>
-      <c r="B36" s="27"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="25"/>
     </row>
     <row r="37" ht="110" customHeight="true">
-      <c r="A37" s="26">
+      <c r="A37" s="24">
         <v>18</v>
       </c>
-      <c r="B37" s="27" t="str">
+      <c r="B37" s="25" t="str">
         <f>data!D21</f>
       </c>
     </row>
     <row r="38" ht="115" customHeight="true">
-      <c r="A38" s="26"/>
-      <c r="B38" s="27"/>
+      <c r="A38" s="24"/>
+      <c r="B38" s="25"/>
     </row>
     <row r="39" ht="110" customHeight="true">
-      <c r="A39" s="26">
+      <c r="A39" s="24">
         <v>19</v>
       </c>
-      <c r="B39" s="27" t="str">
+      <c r="B39" s="25" t="str">
         <f>data!D22</f>
       </c>
     </row>
     <row r="40" ht="115" customHeight="true">
-      <c r="A40" s="26"/>
-      <c r="B40" s="27"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="25"/>
     </row>
     <row r="41" ht="110" customHeight="true">
-      <c r="A41" s="26">
+      <c r="A41" s="24">
         <v>20</v>
       </c>
-      <c r="B41" s="27" t="str">
+      <c r="B41" s="25" t="str">
         <f>data!D23</f>
       </c>
     </row>
     <row r="42" ht="115" customHeight="true">
-      <c r="A42" s="26"/>
-      <c r="B42" s="27"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="25"/>
     </row>
     <row r="43" ht="110" customHeight="true">
-      <c r="A43" s="26">
+      <c r="A43" s="24">
         <v>21</v>
       </c>
-      <c r="B43" s="27" t="str">
+      <c r="B43" s="25" t="str">
         <f>data!D24</f>
       </c>
     </row>
     <row r="44" ht="115" customHeight="true">
-      <c r="A44" s="26"/>
-      <c r="B44" s="27"/>
+      <c r="A44" s="24"/>
+      <c r="B44" s="25"/>
     </row>
     <row r="45" ht="110" customHeight="true">
-      <c r="A45" s="26">
+      <c r="A45" s="24">
         <v>22</v>
       </c>
-      <c r="B45" s="27" t="str">
+      <c r="B45" s="25" t="str">
         <f>data!D25</f>
       </c>
     </row>
     <row r="46" ht="115" customHeight="true">
-      <c r="A46" s="26"/>
-      <c r="B46" s="27"/>
+      <c r="A46" s="24"/>
+      <c r="B46" s="25"/>
     </row>
     <row r="47" ht="110" customHeight="true">
-      <c r="A47" s="26">
+      <c r="A47" s="24">
         <v>23</v>
       </c>
-      <c r="B47" s="27" t="str">
+      <c r="B47" s="25" t="str">
         <f>data!D26</f>
       </c>
     </row>
     <row r="48" ht="115" customHeight="true">
-      <c r="A48" s="26"/>
-      <c r="B48" s="27"/>
+      <c r="A48" s="24"/>
+      <c r="B48" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>